<commit_message>
Testing documents follow the approved proposal
- traceability.md: FR 1-7, NFR 1-7, FR-SPEC/NFR-SPEC, use cases, testing
  objectives, stack and participants mapped to the system and its tests
- Test cases use the proposal's IDs; reply-time target 2 s for 95%;
  new tests for 2G, system health, reports, age range and badge alerts
- UAT participants as in the proposal: ages 15-24 in Kisumu County,
  guardian agreement for 15-17
</commit_message>
<xml_diff>
--- a/docs/testing/MindQuest_testing.xlsx
+++ b/docs/testing/MindQuest_testing.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Bugs" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'System tests'!$A$1:$I$49</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'System tests'!$A$1:$I$54</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="517" uniqueCount="381">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="547" uniqueCount="418">
   <si>
     <t xml:space="preserve">MindQuest – testing workbook (step 12)</t>
   </si>
@@ -61,13 +61,13 @@
     <t xml:space="preserve">Notes</t>
   </si>
   <si>
-    <t xml:space="preserve">• The Covers column uses the proposal's requirement IDs where known (FR 3 gamification, FR 4 articles, FR 5 helplines/crisis, FR 7 and UC-06 reporting, UC-01 chat, UC-02 mood). Check them against the proposal and adjust.</t>
+    <t xml:space="preserve">• The Covers column uses the approved proposal's IDs: FR 1–7 and NFR 1–7 (section 4.1.2), FR-SPEC-01/02 and NFR-SPEC-01/02 (4.3.4), use cases from Figure 4, Table 3 (registration data) and Table 4 (stack). The full mapping is in docs/testing/traceability.md.</t>
   </si>
   <si>
     <t xml:space="preserve">• SUS scoring: odd items score−1, even items 5−score, sum × 2.5 (Brooke, 1996). 68 is the commonly used average; above 68 is above average usability.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Performance targets (replies within 3 s, start within 5 s) are working targets; use the proposal's NFR values if they differ.</t>
+    <t xml:space="preserve">• Reply time target from the proposal (NFR-SPEC-01): under 2 seconds for 95% of messages (ST-20). Start-up within 5 seconds (ST-47) is a working target for NFR 4.</t>
   </si>
   <si>
     <t xml:space="preserve">ID</t>
@@ -103,7 +103,7 @@
     <t xml:space="preserve">Sign-in and onboarding</t>
   </si>
   <si>
-    <t xml:space="preserve">Accounts</t>
+    <t xml:space="preserve">Registration (Table 3), NFR 2</t>
   </si>
   <si>
     <t xml:space="preserve">Fresh install. Welcome → Continue anonymously. Enter a nickname, pick English, tick the privacy box, Let's go.</t>
@@ -118,6 +118,9 @@
     <t xml:space="preserve">ST-02</t>
   </si>
   <si>
+    <t xml:space="preserve">NFR 2 (consent)</t>
+  </si>
+  <si>
     <t xml:space="preserve">On onboarding, leave the privacy box unticked.</t>
   </si>
   <si>
@@ -127,6 +130,9 @@
     <t xml:space="preserve">ST-03</t>
   </si>
   <si>
+    <t xml:space="preserve">User Management module</t>
+  </si>
+  <si>
     <t xml:space="preserve">Create account with a wrong email (abc), then a 5-letter password, then valid details.</t>
   </si>
   <si>
@@ -163,6 +169,9 @@
     <t xml:space="preserve">ST-07</t>
   </si>
   <si>
+    <t xml:space="preserve">NFR 2</t>
+  </si>
+  <si>
     <t xml:space="preserve">Anonymous account: Profile → Sign out.</t>
   </si>
   <si>
@@ -175,9 +184,6 @@
     <t xml:space="preserve">Privacy</t>
   </si>
   <si>
-    <t xml:space="preserve">NFR privacy</t>
-  </si>
-  <si>
     <t xml:space="preserve">Profile → Delete my data → type DELETE (or FUTA) → Delete.</t>
   </si>
   <si>
@@ -190,7 +196,7 @@
     <t xml:space="preserve">Language</t>
   </si>
   <si>
-    <t xml:space="preserve">Bilingual (EN/SW)</t>
+    <t xml:space="preserve">FR 6</t>
   </si>
   <si>
     <t xml:space="preserve">Profile → Language → SW. Visit every tab, then chat "habari".</t>
@@ -205,7 +211,7 @@
     <t xml:space="preserve">Chatbot</t>
   </si>
   <si>
-    <t xml:space="preserve">UC-01</t>
+    <t xml:space="preserve">FR 1, UC 1</t>
   </si>
   <si>
     <t xml:space="preserve">Chat: "Hi, my name is Amani".</t>
@@ -226,6 +232,9 @@
     <t xml:space="preserve">ST-12</t>
   </si>
   <si>
+    <t xml:space="preserve">FR 1, FR 6</t>
+  </si>
+  <si>
     <t xml:space="preserve">Chat in Kiswahili: "nina wasiwasi sana kuhusu kesho".</t>
   </si>
   <si>
@@ -235,6 +244,9 @@
     <t xml:space="preserve">ST-13</t>
   </si>
   <si>
+    <t xml:space="preserve">FR 1, NFR 7</t>
+  </si>
+  <si>
     <t xml:space="preserve">Chat in Sheng/mixed: "niko na stress mbaya sana".</t>
   </si>
   <si>
@@ -256,7 +268,7 @@
     <t xml:space="preserve">Crisis detection</t>
   </si>
   <si>
-    <t xml:space="preserve">FR 5 (crisis support)</t>
+    <t xml:space="preserve">FR 5, FR-SPEC-02, Contact Helpline</t>
   </si>
   <si>
     <t xml:space="preserve">Chat: "I want to end it all".</t>
@@ -268,6 +280,9 @@
     <t xml:space="preserve">ST-16</t>
   </si>
   <si>
+    <t xml:space="preserve">FR 5, FR 6, FR-SPEC-02</t>
+  </si>
+  <si>
     <t xml:space="preserve">Kiswahili profile. Chat: "nataka kujiua".</t>
   </si>
   <si>
@@ -277,6 +292,9 @@
     <t xml:space="preserve">ST-17</t>
   </si>
   <si>
+    <t xml:space="preserve">FR 1</t>
+  </si>
+  <si>
     <t xml:space="preserve">Tap each quick-reply chip.</t>
   </si>
   <si>
@@ -286,7 +304,7 @@
     <t xml:space="preserve">ST-18</t>
   </si>
   <si>
-    <t xml:space="preserve">UC-01, UC-02</t>
+    <t xml:space="preserve">FR 1, FR 2, UC 2</t>
   </si>
   <si>
     <t xml:space="preserve">Chat → "Check in my mood" chip → pick a face.</t>
@@ -310,13 +328,13 @@
     <t xml:space="preserve">Performance</t>
   </si>
   <si>
-    <t xml:space="preserve">NFR performance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Send 5 normal messages; time each reply with a stopwatch (from tapping send to the reply).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Every reply within 3 seconds (write the 5 times in Notes).</t>
+    <t xml:space="preserve">NFR 1, NFR-SPEC-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Normal Wi-Fi or 4G. Send 20 ordinary messages; time each one with a stopwatch from tapping send to the reply appearing. Write the times in Notes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">At least 19 of the 20 replies (95%) within 2 seconds. Also compare with the Reply time tile on the admin Overview.</t>
   </si>
   <si>
     <t xml:space="preserve">ST-21</t>
@@ -325,7 +343,7 @@
     <t xml:space="preserve">Mood tracking</t>
   </si>
   <si>
-    <t xml:space="preserve">UC-02, FR-SPEC-01</t>
+    <t xml:space="preserve">FR 2, UC 2, FR-SPEC-01</t>
   </si>
   <si>
     <t xml:space="preserve">Mood tab: pick Low, tags School + Sleep, a note, Save.</t>
@@ -337,6 +355,9 @@
     <t xml:space="preserve">ST-22</t>
   </si>
   <si>
+    <t xml:space="preserve">FR 3 (reward accuracy)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Check in again the same day.</t>
   </si>
   <si>
@@ -346,6 +367,9 @@
     <t xml:space="preserve">ST-23</t>
   </si>
   <si>
+    <t xml:space="preserve">FR 2, Track Progress</t>
+  </si>
+  <si>
     <t xml:space="preserve">Mood → View mood history. Delete one entry.</t>
   </si>
   <si>
@@ -355,6 +379,9 @@
     <t xml:space="preserve">ST-24</t>
   </si>
   <si>
+    <t xml:space="preserve">FR 2</t>
+  </si>
+  <si>
     <t xml:space="preserve">After 3+ check-ins, open Mood history → Insights.</t>
   </si>
   <si>
@@ -367,7 +394,7 @@
     <t xml:space="preserve">Gamification</t>
   </si>
   <si>
-    <t xml:space="preserve">FR 3, UC-03</t>
+    <t xml:space="preserve">FR 3, Track Progress</t>
   </si>
   <si>
     <t xml:space="preserve">Check in, send a chat message and read an article on the same day.</t>
@@ -379,6 +406,9 @@
     <t xml:space="preserve">ST-26</t>
   </si>
   <si>
+    <t xml:space="preserve">FR 3, Earn Badge</t>
+  </si>
+  <si>
     <t xml:space="preserve">Read and mark 3 different articles.</t>
   </si>
   <si>
@@ -397,6 +427,9 @@
     <t xml:space="preserve">ST-28</t>
   </si>
   <si>
+    <t xml:space="preserve">FR 3 (challenges)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Rewards: look at the weekly quest after check-ins on different days.</t>
   </si>
   <si>
@@ -409,7 +442,7 @@
     <t xml:space="preserve">Learn</t>
   </si>
   <si>
-    <t xml:space="preserve">FR 4 (articles)</t>
+    <t xml:space="preserve">FR 4, View Educational Resources</t>
   </si>
   <si>
     <t xml:space="preserve">Learn: filter by each topic, open an article, switch EN/SW.</t>
@@ -424,7 +457,7 @@
     <t xml:space="preserve">Support</t>
   </si>
   <si>
-    <t xml:space="preserve">FR 5 (helplines)</t>
+    <t xml:space="preserve">FR 5</t>
   </si>
   <si>
     <t xml:space="preserve">Support: start box breathing; do the 5-4-3-2-1 grounding.</t>
@@ -436,6 +469,9 @@
     <t xml:space="preserve">ST-31</t>
   </si>
   <si>
+    <t xml:space="preserve">FR 5, Contact Helpline</t>
+  </si>
+  <si>
     <t xml:space="preserve">Support → Call on a helpline.</t>
   </si>
   <si>
@@ -448,7 +484,7 @@
     <t xml:space="preserve">Offline</t>
   </si>
   <si>
-    <t xml:space="preserve">Step 10</t>
+    <t xml:space="preserve">NFR 6</t>
   </si>
   <si>
     <t xml:space="preserve">Use the app online, close it, turn on aeroplane mode, open it.</t>
@@ -460,6 +496,9 @@
     <t xml:space="preserve">ST-33</t>
   </si>
   <si>
+    <t xml:space="preserve">NFR 6, FR-SPEC-01</t>
+  </si>
+  <si>
     <t xml:space="preserve">Offline: log a mood. Then turn aeroplane mode off and tap Retry.</t>
   </si>
   <si>
@@ -469,7 +508,7 @@
     <t xml:space="preserve">ST-34</t>
   </si>
   <si>
-    <t xml:space="preserve">Step 10, FR 5</t>
+    <t xml:space="preserve">NFR 6, FR 5</t>
   </si>
   <si>
     <t xml:space="preserve">Offline: chat "I want to end it all".</t>
@@ -493,6 +532,9 @@
     <t xml:space="preserve">Reminders</t>
   </si>
   <si>
+    <t xml:space="preserve">Stack: local notifications</t>
+  </si>
+  <si>
     <t xml:space="preserve">Profile → Daily reminder on (allow notifications) → Send a test reminder → tap it.</t>
   </si>
   <si>
@@ -514,7 +556,7 @@
     <t xml:space="preserve">Usability</t>
   </si>
   <si>
-    <t xml:space="preserve">NFR usability</t>
+    <t xml:space="preserve">NFR 4</t>
   </si>
   <si>
     <t xml:space="preserve">Turn on Dark mode; visit every tab.</t>
@@ -535,9 +577,6 @@
     <t xml:space="preserve">ST-40</t>
   </si>
   <si>
-    <t xml:space="preserve">NFR accessibility</t>
-  </si>
-  <si>
     <t xml:space="preserve">Turn on TalkBack; move through Home and the mood faces.</t>
   </si>
   <si>
@@ -550,7 +589,7 @@
     <t xml:space="preserve">Admin dashboard</t>
   </si>
   <si>
-    <t xml:space="preserve">FR 7, UC-06</t>
+    <t xml:space="preserve">FR 7</t>
   </si>
   <si>
     <t xml:space="preserve">Open the admin dashboard; sign in with an admin account, then with a student account.</t>
@@ -562,6 +601,9 @@
     <t xml:space="preserve">ST-42</t>
   </si>
   <si>
+    <t xml:space="preserve">FR 7, Generate Reports</t>
+  </si>
+  <si>
     <t xml:space="preserve">After the tests above, open Overview (7 days).</t>
   </si>
   <si>
@@ -571,6 +613,9 @@
     <t xml:space="preserve">ST-43</t>
   </si>
   <si>
+    <t xml:space="preserve">FR 7, Manage Content</t>
+  </si>
+  <si>
     <t xml:space="preserve">Articles: hide an article, then check the app's Learn tab; publish it again.</t>
   </si>
   <si>
@@ -580,6 +625,9 @@
     <t xml:space="preserve">ST-44</t>
   </si>
   <si>
+    <t xml:space="preserve">FR 7, Manage Content, FR 5</t>
+  </si>
+  <si>
     <t xml:space="preserve">Helplines: mark one verified, then open Support in the app.</t>
   </si>
   <si>
@@ -589,6 +637,9 @@
     <t xml:space="preserve">ST-45</t>
   </si>
   <si>
+    <t xml:space="preserve">View Aggregated Analytics</t>
+  </si>
+  <si>
     <t xml:space="preserve">Team: give a second account Counsellor access; sign in with it.</t>
   </si>
   <si>
@@ -601,7 +652,7 @@
     <t xml:space="preserve">Security</t>
   </si>
   <si>
-    <t xml:space="preserve">NFR security</t>
+    <t xml:space="preserve">NFR 2 (security audit)</t>
   </si>
   <si>
     <t xml:space="preserve">Two phones with two accounts. Log a mood with a note on phone A; open history on phone B.</t>
@@ -625,13 +676,73 @@
     <t xml:space="preserve">Compatibility</t>
   </si>
   <si>
-    <t xml:space="preserve">NFR portability</t>
+    <t xml:space="preserve">NFR 4 (low-end Android)</t>
   </si>
   <si>
     <t xml:space="preserve">Install the release APK on a second Android phone (different brand/version).</t>
   </si>
   <si>
     <t xml:space="preserve">Installs and runs ST-01, ST-11, ST-21 without problems.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ST-49</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NFR 6 (low bandwidth)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phone settings → Mobile network → preferred network 2G (or 3G), Wi-Fi off. Open Home, log a mood, open an article, send a chat message.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Everything works, only slower; nothing crashes; check-ins are saved (on the phone first if the connection drops).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ST-50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monitor System Health, NFR-SPEC-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Overview → System health → Check now. Then stop the Rasa server and Check now again; start it again.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Both rows green with times while running; Chatbot row turns red ("Not working") when Rasa is stopped, and green again after.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ST-51</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generate Reports</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Overview → 7 days → Copy report; paste into Word and into Excel.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Report shows the totals and one row per day; in Excel the day rows split into columns (Data → Text to Columns, comma).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ST-52</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Registration (Table 3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fresh account: on Make it yours, try Let's go without choosing an age range; then choose 18–20.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Let's go stays disabled until an age range is chosen; the admin Overview Age card counts the new student.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ST-53</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FR 3, Earn Badge, stack: notifications</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New account with notifications allowed: send your first chat message; then do your first mood check-in.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"New badge!" pop-up for First Chat, then for First Check-in, and a "New badge" notification for each in the phone's notification shade.</t>
   </si>
   <si>
     <t xml:space="preserve">System test summary</t>
@@ -1765,7 +1876,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
         <v>10</v>
       </c>
@@ -1796,7 +1907,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:I54"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -1870,13 +1981,13 @@
         <v>23</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F3" s="7" t="s">
         <v>27</v>
@@ -1885,21 +1996,21 @@
       <c r="H3" s="7"/>
       <c r="I3" s="7"/>
     </row>
-    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>23</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F4" s="7" t="s">
         <v>27</v>
@@ -1908,21 +2019,21 @@
       <c r="H4" s="7"/>
       <c r="I4" s="7"/>
     </row>
-    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>23</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F5" s="7" t="s">
         <v>27</v>
@@ -1931,21 +2042,21 @@
       <c r="H5" s="7"/>
       <c r="I5" s="7"/>
     </row>
-    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>23</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F6" s="7" t="s">
         <v>27</v>
@@ -1954,21 +2065,21 @@
       <c r="H6" s="7"/>
       <c r="I6" s="7"/>
     </row>
-    <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>23</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F7" s="7" t="s">
         <v>27</v>
@@ -1979,19 +2090,19 @@
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>23</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>24</v>
+        <v>46</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="F8" s="7" t="s">
         <v>27</v>
@@ -2002,19 +2113,19 @@
     </row>
     <row r="9" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="C9" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="B9" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>48</v>
-      </c>
       <c r="D9" s="6" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F9" s="7" t="s">
         <v>27</v>
@@ -2025,19 +2136,19 @@
     </row>
     <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F10" s="7" t="s">
         <v>27</v>
@@ -2048,19 +2159,19 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F11" s="7" t="s">
         <v>27</v>
@@ -2071,19 +2182,19 @@
     </row>
     <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="F12" s="7" t="s">
         <v>27</v>
@@ -2094,19 +2205,19 @@
     </row>
     <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="F13" s="7" t="s">
         <v>27</v>
@@ -2117,19 +2228,19 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>58</v>
+        <v>71</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="F14" s="7" t="s">
         <v>27</v>
@@ -2140,19 +2251,19 @@
     </row>
     <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="F15" s="7" t="s">
         <v>27</v>
@@ -2163,19 +2274,19 @@
     </row>
     <row r="16" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="F16" s="7" t="s">
         <v>27</v>
@@ -2186,19 +2297,19 @@
     </row>
     <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="B17" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="B17" s="6" t="s">
-        <v>74</v>
-      </c>
       <c r="C17" s="6" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="F17" s="7" t="s">
         <v>27</v>
@@ -2209,19 +2320,19 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>58</v>
+        <v>87</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="F18" s="7" t="s">
         <v>27</v>
@@ -2232,19 +2343,19 @@
     </row>
     <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="F19" s="7" t="s">
         <v>27</v>
@@ -2255,19 +2366,19 @@
     </row>
     <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="F20" s="7" t="s">
         <v>27</v>
@@ -2276,21 +2387,21 @@
       <c r="H20" s="7"/>
       <c r="I20" s="7"/>
     </row>
-    <row r="21" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="F21" s="7" t="s">
         <v>27</v>
@@ -2301,19 +2412,19 @@
     </row>
     <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="F22" s="7" t="s">
         <v>27</v>
@@ -2324,19 +2435,19 @@
     </row>
     <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="F23" s="7" t="s">
         <v>27</v>
@@ -2347,19 +2458,19 @@
     </row>
     <row r="24" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="F24" s="7" t="s">
         <v>27</v>
@@ -2370,19 +2481,19 @@
     </row>
     <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>98</v>
+        <v>116</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="F25" s="7" t="s">
         <v>27</v>
@@ -2393,19 +2504,19 @@
     </row>
     <row r="26" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="F26" s="7" t="s">
         <v>27</v>
@@ -2416,19 +2527,19 @@
     </row>
     <row r="27" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>112</v>
+        <v>125</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="F27" s="7" t="s">
         <v>27</v>
@@ -2439,19 +2550,19 @@
     </row>
     <row r="28" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="F28" s="7" t="s">
         <v>27</v>
@@ -2462,19 +2573,19 @@
     </row>
     <row r="29" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>121</v>
+        <v>131</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>112</v>
+        <v>132</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>122</v>
+        <v>133</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="F29" s="7" t="s">
         <v>27</v>
@@ -2483,21 +2594,21 @@
       <c r="H29" s="7"/>
       <c r="I29" s="7"/>
     </row>
-    <row r="30" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>126</v>
+        <v>137</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>127</v>
+        <v>138</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>128</v>
+        <v>139</v>
       </c>
       <c r="F30" s="7" t="s">
         <v>27</v>
@@ -2508,19 +2619,19 @@
     </row>
     <row r="31" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>130</v>
+        <v>141</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>131</v>
+        <v>142</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>133</v>
+        <v>144</v>
       </c>
       <c r="F31" s="7" t="s">
         <v>27</v>
@@ -2529,21 +2640,21 @@
       <c r="H31" s="7"/>
       <c r="I31" s="7"/>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>134</v>
+        <v>145</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>130</v>
+        <v>141</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>131</v>
+        <v>146</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>135</v>
+        <v>147</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>136</v>
+        <v>148</v>
       </c>
       <c r="F32" s="7" t="s">
         <v>27</v>
@@ -2554,19 +2665,19 @@
     </row>
     <row r="33" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>141</v>
+        <v>153</v>
       </c>
       <c r="F33" s="7" t="s">
         <v>27</v>
@@ -2577,19 +2688,19 @@
     </row>
     <row r="34" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>139</v>
+        <v>155</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>143</v>
+        <v>156</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>144</v>
+        <v>157</v>
       </c>
       <c r="F34" s="7" t="s">
         <v>27</v>
@@ -2600,19 +2711,19 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>145</v>
+        <v>158</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>146</v>
+        <v>159</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>147</v>
+        <v>160</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>148</v>
+        <v>161</v>
       </c>
       <c r="F35" s="7" t="s">
         <v>27</v>
@@ -2623,19 +2734,19 @@
     </row>
     <row r="36" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>150</v>
+        <v>163</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>151</v>
+        <v>164</v>
       </c>
       <c r="F36" s="7" t="s">
         <v>27</v>
@@ -2646,19 +2757,19 @@
     </row>
     <row r="37" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="s">
-        <v>152</v>
+        <v>165</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>153</v>
+        <v>166</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>139</v>
+        <v>167</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>154</v>
+        <v>168</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>155</v>
+        <v>169</v>
       </c>
       <c r="F37" s="7" t="s">
         <v>27</v>
@@ -2669,19 +2780,19 @@
     </row>
     <row r="38" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
-        <v>156</v>
+        <v>170</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>153</v>
+        <v>166</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>139</v>
+        <v>167</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>157</v>
+        <v>171</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>158</v>
+        <v>172</v>
       </c>
       <c r="F38" s="7" t="s">
         <v>27</v>
@@ -2692,19 +2803,19 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="s">
-        <v>159</v>
+        <v>173</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>160</v>
+        <v>174</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>161</v>
+        <v>175</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>162</v>
+        <v>176</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>163</v>
+        <v>177</v>
       </c>
       <c r="F39" s="7" t="s">
         <v>27</v>
@@ -2715,19 +2826,19 @@
     </row>
     <row r="40" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="s">
-        <v>164</v>
+        <v>178</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>160</v>
+        <v>174</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>161</v>
+        <v>175</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>165</v>
+        <v>179</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>166</v>
+        <v>180</v>
       </c>
       <c r="F40" s="7" t="s">
         <v>27</v>
@@ -2738,19 +2849,19 @@
     </row>
     <row r="41" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="s">
-        <v>167</v>
+        <v>181</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>160</v>
+        <v>174</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>169</v>
+        <v>182</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>170</v>
+        <v>183</v>
       </c>
       <c r="F41" s="7" t="s">
         <v>27</v>
@@ -2761,19 +2872,19 @@
     </row>
     <row r="42" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="5" t="s">
-        <v>171</v>
+        <v>184</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>172</v>
+        <v>185</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>173</v>
+        <v>186</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>174</v>
+        <v>187</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>175</v>
+        <v>188</v>
       </c>
       <c r="F42" s="7" t="s">
         <v>27</v>
@@ -2784,19 +2895,19 @@
     </row>
     <row r="43" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
-        <v>176</v>
+        <v>189</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>172</v>
+        <v>185</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>173</v>
+        <v>190</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>177</v>
+        <v>191</v>
       </c>
       <c r="E43" s="6" t="s">
-        <v>178</v>
+        <v>192</v>
       </c>
       <c r="F43" s="7" t="s">
         <v>27</v>
@@ -2807,19 +2918,19 @@
     </row>
     <row r="44" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="s">
-        <v>179</v>
+        <v>193</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>172</v>
+        <v>185</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>126</v>
+        <v>194</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>180</v>
+        <v>195</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>181</v>
+        <v>196</v>
       </c>
       <c r="F44" s="7" t="s">
         <v>27</v>
@@ -2830,19 +2941,19 @@
     </row>
     <row r="45" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
-        <v>182</v>
+        <v>197</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>172</v>
+        <v>185</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>131</v>
+        <v>198</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>183</v>
+        <v>199</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>184</v>
+        <v>200</v>
       </c>
       <c r="F45" s="7" t="s">
         <v>27</v>
@@ -2851,21 +2962,21 @@
       <c r="H45" s="7"/>
       <c r="I45" s="7"/>
     </row>
-    <row r="46" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="B46" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="B46" s="6" t="s">
-        <v>172</v>
-      </c>
       <c r="C46" s="6" t="s">
-        <v>173</v>
+        <v>202</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>186</v>
+        <v>203</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>187</v>
+        <v>204</v>
       </c>
       <c r="F46" s="7" t="s">
         <v>27</v>
@@ -2876,19 +2987,19 @@
     </row>
     <row r="47" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="5" t="s">
-        <v>188</v>
+        <v>205</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>189</v>
+        <v>206</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>190</v>
+        <v>207</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>191</v>
+        <v>208</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>192</v>
+        <v>209</v>
       </c>
       <c r="F47" s="7" t="s">
         <v>27</v>
@@ -2899,19 +3010,19 @@
     </row>
     <row r="48" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="5" t="s">
-        <v>193</v>
+        <v>210</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>93</v>
+        <v>175</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>194</v>
+        <v>211</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>195</v>
+        <v>212</v>
       </c>
       <c r="F48" s="7" t="s">
         <v>27</v>
@@ -2922,19 +3033,19 @@
     </row>
     <row r="49" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="5" t="s">
-        <v>196</v>
+        <v>213</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>197</v>
+        <v>214</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>198</v>
+        <v>215</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>199</v>
+        <v>216</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>200</v>
+        <v>217</v>
       </c>
       <c r="F49" s="7" t="s">
         <v>27</v>
@@ -2943,9 +3054,124 @@
       <c r="H49" s="7"/>
       <c r="I49" s="7"/>
     </row>
+    <row r="50" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="B50" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="C50" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="D50" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="E50" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="F50" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G50" s="7"/>
+      <c r="H50" s="7"/>
+      <c r="I50" s="7"/>
+    </row>
+    <row r="51" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="B51" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="C51" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="D51" s="6" t="s">
+        <v>224</v>
+      </c>
+      <c r="E51" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="F51" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G51" s="7"/>
+      <c r="H51" s="7"/>
+      <c r="I51" s="7"/>
+    </row>
+    <row r="52" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="B52" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="C52" s="6" t="s">
+        <v>227</v>
+      </c>
+      <c r="D52" s="6" t="s">
+        <v>228</v>
+      </c>
+      <c r="E52" s="6" t="s">
+        <v>229</v>
+      </c>
+      <c r="F52" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G52" s="7"/>
+      <c r="H52" s="7"/>
+      <c r="I52" s="7"/>
+    </row>
+    <row r="53" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="B53" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C53" s="6" t="s">
+        <v>231</v>
+      </c>
+      <c r="D53" s="6" t="s">
+        <v>232</v>
+      </c>
+      <c r="E53" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="F53" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G53" s="7"/>
+      <c r="H53" s="7"/>
+      <c r="I53" s="7"/>
+    </row>
+    <row r="54" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="B54" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="C54" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="D54" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="E54" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="F54" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G54" s="7"/>
+      <c r="H54" s="7"/>
+      <c r="I54" s="7"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I49"/>
-  <conditionalFormatting sqref="F2:F49">
+  <autoFilter ref="A1:I54"/>
+  <conditionalFormatting sqref="F2:F54">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
       <formula>"Pass"</formula>
     </cfRule>
@@ -2957,7 +3183,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F2:F49" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F2:F54" type="list">
       <formula1>"Pass,Fail,Blocked,Not run"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2988,7 +3214,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>201</v>
+        <v>238</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2996,33 +3222,33 @@
         <v>18</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>202</v>
+        <v>239</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>203</v>
+        <v>240</v>
       </c>
       <c r="B4" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$F$2:$F$49,A4)</f>
+        <f aca="false">COUNTIF('System tests'!$F$2:$F$54,A4)</f>
         <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>204</v>
+        <v>241</v>
       </c>
       <c r="B5" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$F$2:$F$49,A5)</f>
+        <f aca="false">COUNTIF('System tests'!$F$2:$F$54,A5)</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>205</v>
+        <v>242</v>
       </c>
       <c r="B6" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$F$2:$F$49,A6)</f>
+        <f aca="false">COUNTIF('System tests'!$F$2:$F$54,A6)</f>
         <v>0</v>
       </c>
     </row>
@@ -3031,22 +3257,22 @@
         <v>27</v>
       </c>
       <c r="B7" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$F$2:$F$49,A7)</f>
-        <v>48</v>
+        <f aca="false">COUNTIF('System tests'!$F$2:$F$54,A7)</f>
+        <v>53</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>206</v>
+        <v>243</v>
       </c>
       <c r="B8" s="5" t="n">
         <f aca="false">SUM(B4:B7)</f>
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>207</v>
+        <v>244</v>
       </c>
       <c r="B9" s="9" t="str">
         <f aca="false">IF(B4+B5+B6=0,"-",B4/(B4+B5+B6))</f>
@@ -3058,22 +3284,22 @@
         <v>14</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>202</v>
+        <v>239</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>203</v>
+        <v>240</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>204</v>
+        <v>241</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>205</v>
+        <v>242</v>
       </c>
       <c r="F11" s="4" t="s">
         <v>27</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>208</v>
+        <v>245</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3081,24 +3307,24 @@
         <v>23</v>
       </c>
       <c r="B12" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$49,A12)</f>
-        <v>7</v>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$54,A12)</f>
+        <v>8</v>
       </c>
       <c r="C12" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A12,'System tests'!$F$2:$F$49,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A12,'System tests'!$F$2:$F$54,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D12" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A12,'System tests'!$F$2:$F$49,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A12,'System tests'!$F$2:$F$54,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E12" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A12,'System tests'!$F$2:$F$49,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A12,'System tests'!$F$2:$F$54,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F12" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A12,'System tests'!$F$2:$F$49,"Not run")</f>
-        <v>7</v>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A12,'System tests'!$F$2:$F$54,"Not run")</f>
+        <v>8</v>
       </c>
       <c r="G12" s="10" t="str">
         <f aca="false">IF(C12+D12+E12=0,"-",C12/(C12+D12+E12))</f>
@@ -3107,26 +3333,26 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B13" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$49,A13)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$54,A13)</f>
         <v>1</v>
       </c>
       <c r="C13" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A13,'System tests'!$F$2:$F$49,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A13,'System tests'!$F$2:$F$54,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D13" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A13,'System tests'!$F$2:$F$49,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A13,'System tests'!$F$2:$F$54,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E13" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A13,'System tests'!$F$2:$F$49,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A13,'System tests'!$F$2:$F$54,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F13" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A13,'System tests'!$F$2:$F$49,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A13,'System tests'!$F$2:$F$54,"Not run")</f>
         <v>1</v>
       </c>
       <c r="G13" s="10" t="str">
@@ -3136,26 +3362,26 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B14" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$49,A14)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$54,A14)</f>
         <v>1</v>
       </c>
       <c r="C14" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A14,'System tests'!$F$2:$F$49,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A14,'System tests'!$F$2:$F$54,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D14" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A14,'System tests'!$F$2:$F$49,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A14,'System tests'!$F$2:$F$54,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E14" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A14,'System tests'!$F$2:$F$49,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A14,'System tests'!$F$2:$F$54,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F14" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A14,'System tests'!$F$2:$F$49,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A14,'System tests'!$F$2:$F$54,"Not run")</f>
         <v>1</v>
       </c>
       <c r="G14" s="10" t="str">
@@ -3165,26 +3391,26 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B15" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$49,A15)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$54,A15)</f>
         <v>8</v>
       </c>
       <c r="C15" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A15,'System tests'!$F$2:$F$49,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A15,'System tests'!$F$2:$F$54,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D15" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A15,'System tests'!$F$2:$F$49,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A15,'System tests'!$F$2:$F$54,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E15" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A15,'System tests'!$F$2:$F$49,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A15,'System tests'!$F$2:$F$54,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F15" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A15,'System tests'!$F$2:$F$49,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A15,'System tests'!$F$2:$F$54,"Not run")</f>
         <v>8</v>
       </c>
       <c r="G15" s="10" t="str">
@@ -3194,26 +3420,26 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="B16" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$49,A16)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$54,A16)</f>
         <v>2</v>
       </c>
       <c r="C16" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A16,'System tests'!$F$2:$F$49,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A16,'System tests'!$F$2:$F$54,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D16" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A16,'System tests'!$F$2:$F$49,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A16,'System tests'!$F$2:$F$54,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E16" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A16,'System tests'!$F$2:$F$49,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A16,'System tests'!$F$2:$F$54,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F16" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A16,'System tests'!$F$2:$F$49,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A16,'System tests'!$F$2:$F$54,"Not run")</f>
         <v>2</v>
       </c>
       <c r="G16" s="10" t="str">
@@ -3223,26 +3449,26 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="B17" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$49,A17)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$54,A17)</f>
         <v>2</v>
       </c>
       <c r="C17" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A17,'System tests'!$F$2:$F$49,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A17,'System tests'!$F$2:$F$54,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D17" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A17,'System tests'!$F$2:$F$49,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A17,'System tests'!$F$2:$F$54,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E17" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A17,'System tests'!$F$2:$F$49,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A17,'System tests'!$F$2:$F$54,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F17" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A17,'System tests'!$F$2:$F$49,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A17,'System tests'!$F$2:$F$54,"Not run")</f>
         <v>2</v>
       </c>
       <c r="G17" s="10" t="str">
@@ -3252,26 +3478,26 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="B18" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$49,A18)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$54,A18)</f>
         <v>4</v>
       </c>
       <c r="C18" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A18,'System tests'!$F$2:$F$49,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A18,'System tests'!$F$2:$F$54,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D18" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A18,'System tests'!$F$2:$F$49,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A18,'System tests'!$F$2:$F$54,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E18" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A18,'System tests'!$F$2:$F$49,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A18,'System tests'!$F$2:$F$54,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F18" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A18,'System tests'!$F$2:$F$49,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A18,'System tests'!$F$2:$F$54,"Not run")</f>
         <v>4</v>
       </c>
       <c r="G18" s="10" t="str">
@@ -3281,27 +3507,27 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="B19" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$49,A19)</f>
-        <v>4</v>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$54,A19)</f>
+        <v>5</v>
       </c>
       <c r="C19" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A19,'System tests'!$F$2:$F$49,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A19,'System tests'!$F$2:$F$54,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D19" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A19,'System tests'!$F$2:$F$49,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A19,'System tests'!$F$2:$F$54,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E19" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A19,'System tests'!$F$2:$F$49,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A19,'System tests'!$F$2:$F$54,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F19" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A19,'System tests'!$F$2:$F$49,"Not run")</f>
-        <v>4</v>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A19,'System tests'!$F$2:$F$54,"Not run")</f>
+        <v>5</v>
       </c>
       <c r="G19" s="10" t="str">
         <f aca="false">IF(C19+D19+E19=0,"-",C19/(C19+D19+E19))</f>
@@ -3310,26 +3536,26 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="B20" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$49,A20)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$54,A20)</f>
         <v>1</v>
       </c>
       <c r="C20" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A20,'System tests'!$F$2:$F$49,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A20,'System tests'!$F$2:$F$54,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D20" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A20,'System tests'!$F$2:$F$49,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A20,'System tests'!$F$2:$F$54,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E20" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A20,'System tests'!$F$2:$F$49,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A20,'System tests'!$F$2:$F$54,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F20" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A20,'System tests'!$F$2:$F$49,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A20,'System tests'!$F$2:$F$54,"Not run")</f>
         <v>1</v>
       </c>
       <c r="G20" s="10" t="str">
@@ -3339,26 +3565,26 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>130</v>
+        <v>141</v>
       </c>
       <c r="B21" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$49,A21)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$54,A21)</f>
         <v>2</v>
       </c>
       <c r="C21" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A21,'System tests'!$F$2:$F$49,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A21,'System tests'!$F$2:$F$54,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D21" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A21,'System tests'!$F$2:$F$49,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A21,'System tests'!$F$2:$F$54,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E21" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A21,'System tests'!$F$2:$F$49,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A21,'System tests'!$F$2:$F$54,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F21" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A21,'System tests'!$F$2:$F$49,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A21,'System tests'!$F$2:$F$54,"Not run")</f>
         <v>2</v>
       </c>
       <c r="G21" s="10" t="str">
@@ -3368,27 +3594,27 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="B22" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$49,A22)</f>
-        <v>4</v>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$54,A22)</f>
+        <v>5</v>
       </c>
       <c r="C22" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A22,'System tests'!$F$2:$F$49,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A22,'System tests'!$F$2:$F$54,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D22" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A22,'System tests'!$F$2:$F$49,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A22,'System tests'!$F$2:$F$54,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E22" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A22,'System tests'!$F$2:$F$49,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A22,'System tests'!$F$2:$F$54,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F22" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A22,'System tests'!$F$2:$F$49,"Not run")</f>
-        <v>4</v>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A22,'System tests'!$F$2:$F$54,"Not run")</f>
+        <v>5</v>
       </c>
       <c r="G22" s="10" t="str">
         <f aca="false">IF(C22+D22+E22=0,"-",C22/(C22+D22+E22))</f>
@@ -3397,26 +3623,26 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>153</v>
+        <v>166</v>
       </c>
       <c r="B23" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$49,A23)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$54,A23)</f>
         <v>2</v>
       </c>
       <c r="C23" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A23,'System tests'!$F$2:$F$49,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A23,'System tests'!$F$2:$F$54,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D23" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A23,'System tests'!$F$2:$F$49,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A23,'System tests'!$F$2:$F$54,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E23" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A23,'System tests'!$F$2:$F$49,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A23,'System tests'!$F$2:$F$54,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F23" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A23,'System tests'!$F$2:$F$49,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A23,'System tests'!$F$2:$F$54,"Not run")</f>
         <v>2</v>
       </c>
       <c r="G23" s="10" t="str">
@@ -3426,26 +3652,26 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>160</v>
+        <v>174</v>
       </c>
       <c r="B24" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$49,A24)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$54,A24)</f>
         <v>3</v>
       </c>
       <c r="C24" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A24,'System tests'!$F$2:$F$49,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A24,'System tests'!$F$2:$F$54,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D24" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A24,'System tests'!$F$2:$F$49,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A24,'System tests'!$F$2:$F$54,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E24" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A24,'System tests'!$F$2:$F$49,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A24,'System tests'!$F$2:$F$54,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F24" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A24,'System tests'!$F$2:$F$49,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A24,'System tests'!$F$2:$F$54,"Not run")</f>
         <v>3</v>
       </c>
       <c r="G24" s="10" t="str">
@@ -3455,27 +3681,27 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>172</v>
+        <v>185</v>
       </c>
       <c r="B25" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$49,A25)</f>
-        <v>5</v>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$54,A25)</f>
+        <v>7</v>
       </c>
       <c r="C25" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A25,'System tests'!$F$2:$F$49,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A25,'System tests'!$F$2:$F$54,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D25" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A25,'System tests'!$F$2:$F$49,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A25,'System tests'!$F$2:$F$54,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E25" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A25,'System tests'!$F$2:$F$49,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A25,'System tests'!$F$2:$F$54,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F25" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A25,'System tests'!$F$2:$F$49,"Not run")</f>
-        <v>5</v>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A25,'System tests'!$F$2:$F$54,"Not run")</f>
+        <v>7</v>
       </c>
       <c r="G25" s="10" t="str">
         <f aca="false">IF(C25+D25+E25=0,"-",C25/(C25+D25+E25))</f>
@@ -3484,26 +3710,26 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>189</v>
+        <v>206</v>
       </c>
       <c r="B26" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$49,A26)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$54,A26)</f>
         <v>1</v>
       </c>
       <c r="C26" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A26,'System tests'!$F$2:$F$49,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A26,'System tests'!$F$2:$F$54,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D26" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A26,'System tests'!$F$2:$F$49,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A26,'System tests'!$F$2:$F$54,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E26" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A26,'System tests'!$F$2:$F$49,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A26,'System tests'!$F$2:$F$54,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F26" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A26,'System tests'!$F$2:$F$49,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A26,'System tests'!$F$2:$F$54,"Not run")</f>
         <v>1</v>
       </c>
       <c r="G26" s="10" t="str">
@@ -3513,26 +3739,26 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>197</v>
+        <v>214</v>
       </c>
       <c r="B27" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$49,A27)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$54,A27)</f>
         <v>1</v>
       </c>
       <c r="C27" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A27,'System tests'!$F$2:$F$49,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A27,'System tests'!$F$2:$F$54,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D27" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A27,'System tests'!$F$2:$F$49,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A27,'System tests'!$F$2:$F$54,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E27" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A27,'System tests'!$F$2:$F$49,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A27,'System tests'!$F$2:$F$54,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F27" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$49,$A27,'System tests'!$F$2:$F$49,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A27,'System tests'!$F$2:$F$54,"Not run")</f>
         <v>1</v>
       </c>
       <c r="G27" s="10" t="str">
@@ -3572,50 +3798,50 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>209</v>
+        <v>246</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>210</v>
+        <v>247</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>211</v>
+        <v>248</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>212</v>
+        <v>249</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>213</v>
+        <v>250</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>214</v>
+        <v>251</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>215</v>
+        <v>252</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>216</v>
+        <v>253</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>217</v>
+        <v>254</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>218</v>
+        <v>255</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>219</v>
+        <v>256</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>220</v>
+        <v>257</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>221</v>
+        <v>258</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>222</v>
+        <v>259</v>
       </c>
       <c r="D4" s="7"/>
       <c r="E4" s="7"/>
@@ -3636,13 +3862,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>223</v>
+        <v>260</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>224</v>
+        <v>261</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>225</v>
+        <v>262</v>
       </c>
       <c r="D5" s="7"/>
       <c r="E5" s="7"/>
@@ -3663,13 +3889,13 @@
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>226</v>
+        <v>263</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>227</v>
+        <v>264</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>228</v>
+        <v>265</v>
       </c>
       <c r="D6" s="7"/>
       <c r="E6" s="7"/>
@@ -3690,13 +3916,13 @@
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>229</v>
+        <v>266</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>230</v>
+        <v>267</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>231</v>
+        <v>268</v>
       </c>
       <c r="D7" s="7"/>
       <c r="E7" s="7"/>
@@ -3717,13 +3943,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>232</v>
+        <v>269</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>233</v>
+        <v>270</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>234</v>
+        <v>271</v>
       </c>
       <c r="D8" s="7"/>
       <c r="E8" s="7"/>
@@ -3744,13 +3970,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>235</v>
+        <v>272</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>236</v>
+        <v>273</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>237</v>
+        <v>274</v>
       </c>
       <c r="D9" s="7"/>
       <c r="E9" s="7"/>
@@ -3771,13 +3997,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>238</v>
+        <v>275</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>239</v>
+        <v>276</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>240</v>
+        <v>277</v>
       </c>
       <c r="D10" s="7"/>
       <c r="E10" s="7"/>
@@ -3798,13 +4024,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>241</v>
+        <v>278</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>242</v>
+        <v>279</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>243</v>
+        <v>280</v>
       </c>
       <c r="D11" s="7"/>
       <c r="E11" s="7"/>
@@ -3825,7 +4051,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="12" t="s">
-        <v>244</v>
+        <v>281</v>
       </c>
     </row>
   </sheetData>
@@ -3856,53 +4082,53 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>245</v>
+        <v>282</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>246</v>
+        <v>283</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>247</v>
+        <v>284</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>248</v>
+        <v>285</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>249</v>
+        <v>286</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>250</v>
+        <v>287</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>251</v>
+        <v>288</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>252</v>
+        <v>289</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>253</v>
+        <v>290</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>254</v>
+        <v>291</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>255</v>
+        <v>292</v>
       </c>
       <c r="K3" s="4" t="s">
-        <v>256</v>
+        <v>293</v>
       </c>
       <c r="L3" s="4" t="s">
-        <v>257</v>
+        <v>294</v>
       </c>
       <c r="N3" s="11" t="s">
-        <v>258</v>
+        <v>295</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>259</v>
+        <v>296</v>
       </c>
       <c r="B4" s="13" t="n">
         <v>4</v>
@@ -3939,7 +4165,7 @@
         <v>80</v>
       </c>
       <c r="N4" s="5" t="s">
-        <v>260</v>
+        <v>297</v>
       </c>
       <c r="O4" s="14" t="n">
         <f aca="false">COUNT(L5:L34)</f>
@@ -3948,7 +4174,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>261</v>
+        <v>298</v>
       </c>
       <c r="B5" s="7"/>
       <c r="C5" s="7"/>
@@ -3965,7 +4191,7 @@
         <v/>
       </c>
       <c r="N5" s="5" t="s">
-        <v>262</v>
+        <v>299</v>
       </c>
       <c r="O5" s="15" t="str">
         <f aca="false">IF(COUNT(L5:L34)=0,"-",AVERAGE(L5:L34))</f>
@@ -3974,7 +4200,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>263</v>
+        <v>300</v>
       </c>
       <c r="B6" s="7"/>
       <c r="C6" s="7"/>
@@ -3991,7 +4217,7 @@
         <v/>
       </c>
       <c r="N6" s="5" t="s">
-        <v>264</v>
+        <v>301</v>
       </c>
       <c r="O6" s="15" t="str">
         <f aca="false">IF(COUNT(L5:L34)=0,"-",MEDIAN(L5:L34))</f>
@@ -4000,7 +4226,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>265</v>
+        <v>302</v>
       </c>
       <c r="B7" s="7"/>
       <c r="C7" s="7"/>
@@ -4017,7 +4243,7 @@
         <v/>
       </c>
       <c r="N7" s="5" t="s">
-        <v>266</v>
+        <v>303</v>
       </c>
       <c r="O7" s="15" t="str">
         <f aca="false">IF(COUNT(L5:L34)&lt;2,"-",STDEV(L5:L34))</f>
@@ -4026,7 +4252,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>267</v>
+        <v>304</v>
       </c>
       <c r="B8" s="7"/>
       <c r="C8" s="7"/>
@@ -4043,7 +4269,7 @@
         <v/>
       </c>
       <c r="N8" s="5" t="s">
-        <v>268</v>
+        <v>305</v>
       </c>
       <c r="O8" s="15" t="str">
         <f aca="false">IF(COUNT(L5:L34)=0,"-",MIN(L5:L34))</f>
@@ -4052,7 +4278,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>269</v>
+        <v>306</v>
       </c>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
@@ -4069,7 +4295,7 @@
         <v/>
       </c>
       <c r="N9" s="5" t="s">
-        <v>270</v>
+        <v>307</v>
       </c>
       <c r="O9" s="15" t="str">
         <f aca="false">IF(COUNT(L5:L34)=0,"-",MAX(L5:L34))</f>
@@ -4078,7 +4304,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>271</v>
+        <v>308</v>
       </c>
       <c r="B10" s="7"/>
       <c r="C10" s="7"/>
@@ -4095,7 +4321,7 @@
         <v/>
       </c>
       <c r="N10" s="5" t="s">
-        <v>272</v>
+        <v>309</v>
       </c>
       <c r="O10" s="16" t="str">
         <f aca="false">IF(COUNT(L5:L34)=0,"-",IF(AVERAGE(L5:L34)&gt;68,"Yes","No"))</f>
@@ -4104,7 +4330,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>273</v>
+        <v>310</v>
       </c>
       <c r="B11" s="7"/>
       <c r="C11" s="7"/>
@@ -4123,7 +4349,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>274</v>
+        <v>311</v>
       </c>
       <c r="B12" s="7"/>
       <c r="C12" s="7"/>
@@ -4140,12 +4366,12 @@
         <v/>
       </c>
       <c r="N12" s="11" t="s">
-        <v>275</v>
+        <v>312</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>276</v>
+        <v>313</v>
       </c>
       <c r="B13" s="7"/>
       <c r="C13" s="7"/>
@@ -4162,12 +4388,12 @@
         <v/>
       </c>
       <c r="N13" s="17" t="s">
-        <v>277</v>
+        <v>314</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>278</v>
+        <v>315</v>
       </c>
       <c r="B14" s="7"/>
       <c r="C14" s="7"/>
@@ -4184,12 +4410,12 @@
         <v/>
       </c>
       <c r="N14" s="17" t="s">
-        <v>279</v>
+        <v>316</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>280</v>
+        <v>317</v>
       </c>
       <c r="B15" s="7"/>
       <c r="C15" s="7"/>
@@ -4206,12 +4432,12 @@
         <v/>
       </c>
       <c r="N15" s="17" t="s">
-        <v>281</v>
+        <v>318</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>282</v>
+        <v>319</v>
       </c>
       <c r="B16" s="7"/>
       <c r="C16" s="7"/>
@@ -4228,12 +4454,12 @@
         <v/>
       </c>
       <c r="N16" s="17" t="s">
-        <v>283</v>
+        <v>320</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>284</v>
+        <v>321</v>
       </c>
       <c r="B17" s="7"/>
       <c r="C17" s="7"/>
@@ -4250,12 +4476,12 @@
         <v/>
       </c>
       <c r="N17" s="17" t="s">
-        <v>285</v>
+        <v>322</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>286</v>
+        <v>323</v>
       </c>
       <c r="B18" s="7"/>
       <c r="C18" s="7"/>
@@ -4272,12 +4498,12 @@
         <v/>
       </c>
       <c r="N18" s="17" t="s">
-        <v>287</v>
+        <v>324</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>288</v>
+        <v>325</v>
       </c>
       <c r="B19" s="7"/>
       <c r="C19" s="7"/>
@@ -4294,12 +4520,12 @@
         <v/>
       </c>
       <c r="N19" s="17" t="s">
-        <v>289</v>
+        <v>326</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>290</v>
+        <v>327</v>
       </c>
       <c r="B20" s="7"/>
       <c r="C20" s="7"/>
@@ -4316,12 +4542,12 @@
         <v/>
       </c>
       <c r="N20" s="17" t="s">
-        <v>291</v>
+        <v>328</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>292</v>
+        <v>329</v>
       </c>
       <c r="B21" s="7"/>
       <c r="C21" s="7"/>
@@ -4338,12 +4564,12 @@
         <v/>
       </c>
       <c r="N21" s="17" t="s">
-        <v>293</v>
+        <v>330</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>294</v>
+        <v>331</v>
       </c>
       <c r="B22" s="7"/>
       <c r="C22" s="7"/>
@@ -4360,12 +4586,12 @@
         <v/>
       </c>
       <c r="N22" s="17" t="s">
-        <v>295</v>
+        <v>332</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>296</v>
+        <v>333</v>
       </c>
       <c r="B23" s="7"/>
       <c r="C23" s="7"/>
@@ -4384,7 +4610,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>297</v>
+        <v>334</v>
       </c>
       <c r="B24" s="7"/>
       <c r="C24" s="7"/>
@@ -4403,7 +4629,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>298</v>
+        <v>335</v>
       </c>
       <c r="B25" s="7"/>
       <c r="C25" s="7"/>
@@ -4422,7 +4648,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>299</v>
+        <v>336</v>
       </c>
       <c r="B26" s="7"/>
       <c r="C26" s="7"/>
@@ -4441,7 +4667,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
-        <v>300</v>
+        <v>337</v>
       </c>
       <c r="B27" s="7"/>
       <c r="C27" s="7"/>
@@ -4460,7 +4686,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
-        <v>301</v>
+        <v>338</v>
       </c>
       <c r="B28" s="7"/>
       <c r="C28" s="7"/>
@@ -4479,7 +4705,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
-        <v>302</v>
+        <v>339</v>
       </c>
       <c r="B29" s="7"/>
       <c r="C29" s="7"/>
@@ -4498,7 +4724,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
-        <v>303</v>
+        <v>340</v>
       </c>
       <c r="B30" s="7"/>
       <c r="C30" s="7"/>
@@ -4517,7 +4743,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
-        <v>304</v>
+        <v>341</v>
       </c>
       <c r="B31" s="7"/>
       <c r="C31" s="7"/>
@@ -4536,7 +4762,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
-        <v>305</v>
+        <v>342</v>
       </c>
       <c r="B32" s="7"/>
       <c r="C32" s="7"/>
@@ -4555,7 +4781,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
-        <v>306</v>
+        <v>343</v>
       </c>
       <c r="B33" s="7"/>
       <c r="C33" s="7"/>
@@ -4574,7 +4800,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
-        <v>307</v>
+        <v>344</v>
       </c>
       <c r="B34" s="7"/>
       <c r="C34" s="7"/>
@@ -4626,47 +4852,47 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>308</v>
+        <v>345</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>309</v>
+        <v>346</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>310</v>
+        <v>347</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>311</v>
+        <v>348</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>312</v>
+        <v>349</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>313</v>
+        <v>350</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>314</v>
+        <v>351</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>315</v>
+        <v>352</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>217</v>
+        <v>254</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>316</v>
+        <v>353</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>317</v>
+        <v>354</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>318</v>
+        <v>355</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>319</v>
+        <v>356</v>
       </c>
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>
@@ -4688,10 +4914,10 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>320</v>
+        <v>357</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>321</v>
+        <v>358</v>
       </c>
       <c r="C5" s="7"/>
       <c r="D5" s="7"/>
@@ -4713,10 +4939,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>322</v>
+        <v>359</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>323</v>
+        <v>360</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="7"/>
@@ -4738,10 +4964,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>324</v>
+        <v>361</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>325</v>
+        <v>362</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
@@ -4763,10 +4989,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>326</v>
+        <v>363</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>327</v>
+        <v>364</v>
       </c>
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
@@ -4788,10 +5014,10 @@
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>328</v>
+        <v>365</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>329</v>
+        <v>366</v>
       </c>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
@@ -4813,10 +5039,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>330</v>
+        <v>367</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>331</v>
+        <v>368</v>
       </c>
       <c r="C10" s="7"/>
       <c r="D10" s="7"/>
@@ -4838,10 +5064,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>332</v>
+        <v>369</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>333</v>
+        <v>370</v>
       </c>
       <c r="C11" s="7"/>
       <c r="D11" s="7"/>
@@ -4863,10 +5089,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>334</v>
+        <v>371</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>335</v>
+        <v>372</v>
       </c>
       <c r="C12" s="7"/>
       <c r="D12" s="7"/>
@@ -4888,10 +5114,10 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>336</v>
+        <v>373</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>337</v>
+        <v>374</v>
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="7"/>
@@ -4913,7 +5139,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="12" t="s">
-        <v>338</v>
+        <v>375</v>
       </c>
     </row>
   </sheetData>
@@ -4945,53 +5171,53 @@
   <sheetData>
     <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>339</v>
+        <v>376</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>340</v>
+        <v>377</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>341</v>
+        <v>378</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>342</v>
+        <v>379</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>343</v>
+        <v>380</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>344</v>
+        <v>381</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>345</v>
+        <v>382</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="13" t="s">
-        <v>259</v>
+        <v>296</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>164</v>
+        <v>178</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>346</v>
+        <v>383</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>347</v>
+        <v>384</v>
       </c>
       <c r="E2" s="13" t="s">
-        <v>348</v>
+        <v>385</v>
       </c>
       <c r="F2" s="13" t="s">
-        <v>349</v>
+        <v>386</v>
       </c>
       <c r="G2" s="13" t="s">
-        <v>350</v>
+        <v>387</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>351</v>
+        <v>388</v>
       </c>
       <c r="B3" s="7"/>
       <c r="C3" s="7"/>
@@ -5002,7 +5228,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>352</v>
+        <v>389</v>
       </c>
       <c r="B4" s="7"/>
       <c r="C4" s="7"/>
@@ -5013,7 +5239,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>353</v>
+        <v>390</v>
       </c>
       <c r="B5" s="7"/>
       <c r="C5" s="7"/>
@@ -5024,7 +5250,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>354</v>
+        <v>391</v>
       </c>
       <c r="B6" s="7"/>
       <c r="C6" s="7"/>
@@ -5035,7 +5261,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>355</v>
+        <v>392</v>
       </c>
       <c r="B7" s="7"/>
       <c r="C7" s="7"/>
@@ -5046,7 +5272,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>356</v>
+        <v>393</v>
       </c>
       <c r="B8" s="7"/>
       <c r="C8" s="7"/>
@@ -5057,7 +5283,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>357</v>
+        <v>394</v>
       </c>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
@@ -5068,7 +5294,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>358</v>
+        <v>395</v>
       </c>
       <c r="B10" s="7"/>
       <c r="C10" s="7"/>
@@ -5079,7 +5305,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>359</v>
+        <v>396</v>
       </c>
       <c r="B11" s="7"/>
       <c r="C11" s="7"/>
@@ -5090,7 +5316,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>360</v>
+        <v>397</v>
       </c>
       <c r="B12" s="7"/>
       <c r="C12" s="7"/>
@@ -5101,7 +5327,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>361</v>
+        <v>398</v>
       </c>
       <c r="B13" s="7"/>
       <c r="C13" s="7"/>
@@ -5112,7 +5338,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>362</v>
+        <v>399</v>
       </c>
       <c r="B14" s="7"/>
       <c r="C14" s="7"/>
@@ -5123,7 +5349,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>363</v>
+        <v>400</v>
       </c>
       <c r="B15" s="7"/>
       <c r="C15" s="7"/>
@@ -5134,7 +5360,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>364</v>
+        <v>401</v>
       </c>
       <c r="B16" s="7"/>
       <c r="C16" s="7"/>
@@ -5145,7 +5371,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>365</v>
+        <v>402</v>
       </c>
       <c r="B17" s="7"/>
       <c r="C17" s="7"/>
@@ -5156,7 +5382,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>366</v>
+        <v>403</v>
       </c>
       <c r="B18" s="7"/>
       <c r="C18" s="7"/>
@@ -5167,7 +5393,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>367</v>
+        <v>404</v>
       </c>
       <c r="B19" s="7"/>
       <c r="C19" s="7"/>
@@ -5178,7 +5404,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>368</v>
+        <v>405</v>
       </c>
       <c r="B20" s="7"/>
       <c r="C20" s="7"/>
@@ -5189,7 +5415,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>369</v>
+        <v>406</v>
       </c>
       <c r="B21" s="7"/>
       <c r="C21" s="7"/>
@@ -5200,7 +5426,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>370</v>
+        <v>407</v>
       </c>
       <c r="B22" s="7"/>
       <c r="C22" s="7"/>
@@ -5211,7 +5437,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>371</v>
+        <v>408</v>
       </c>
       <c r="B23" s="7"/>
       <c r="C23" s="7"/>
@@ -5222,7 +5448,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>372</v>
+        <v>409</v>
       </c>
       <c r="B24" s="7"/>
       <c r="C24" s="7"/>
@@ -5233,7 +5459,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>373</v>
+        <v>410</v>
       </c>
       <c r="B25" s="7"/>
       <c r="C25" s="7"/>
@@ -5244,7 +5470,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>374</v>
+        <v>411</v>
       </c>
       <c r="B26" s="7"/>
       <c r="C26" s="7"/>
@@ -5255,7 +5481,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>375</v>
+        <v>412</v>
       </c>
       <c r="B27" s="7"/>
       <c r="C27" s="7"/>
@@ -5266,7 +5492,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
-        <v>376</v>
+        <v>413</v>
       </c>
       <c r="B28" s="7"/>
       <c r="C28" s="7"/>
@@ -5277,7 +5503,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>377</v>
+        <v>414</v>
       </c>
       <c r="B29" s="7"/>
       <c r="C29" s="7"/>
@@ -5288,7 +5514,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
-        <v>378</v>
+        <v>415</v>
       </c>
       <c r="B30" s="7"/>
       <c r="C30" s="7"/>
@@ -5299,7 +5525,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
-        <v>379</v>
+        <v>416</v>
       </c>
       <c r="B31" s="7"/>
       <c r="C31" s="7"/>
@@ -5310,7 +5536,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
-        <v>380</v>
+        <v>417</v>
       </c>
       <c r="B32" s="7"/>
       <c r="C32" s="7"/>

</xml_diff>

<commit_message>
Testing workbook: cases for rest days, outfits and challenges
</commit_message>
<xml_diff>
--- a/docs/testing/MindQuest_testing.xlsx
+++ b/docs/testing/MindQuest_testing.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Bugs" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'System tests'!$A$1:$I$54</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'System tests'!$A$1:$I$62</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="547" uniqueCount="418">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="605" uniqueCount="457">
   <si>
     <t xml:space="preserve">MindQuest – testing workbook (step 12)</t>
   </si>
@@ -745,6 +745,93 @@
     <t xml:space="preserve">"New badge!" pop-up for First Chat, then for First Check-in, and a "New badge" notification for each in the phone's notification shade.</t>
   </si>
   <si>
+    <t xml:space="preserve">ST-54</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FR 3 (streaks)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check in on two days in a row (e.g. Mon, Tue). Skip the next day. On the day after, open Home before checking in; then check in.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Before: "Yesterday was your rest day. Check in today to keep your streak!" and the streak still 2. After: 3-day streak, the line says the rest day is used this week, and the 3-Day Streak badge pop-up.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ST-55</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FR 3 (streaks, reward accuracy)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In the same week as ST-54, skip one more day, then check in.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The streak starts again at 1 (only one rest day per week); XP, level and badges stay.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ST-56</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FR 3 (rewards)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New account: earn 50 XP (e.g. check in, read articles, chat) until Level 2, then open Home.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Level up!" with Chipu wearing the daisy; Put it on → Chipu wears the daisy on Home, Rewards and next to his chat messages.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ST-57</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rewards → Chipu's wardrobe: tap a locked outfit, then an unlocked one, then Just Chipu.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Locked ones show "Level N" with a lock and nothing happens; an unlocked one is worn at once (message "Chipu is wearing …"); Just Chipu removes it. The choice is the same after closing and opening the app.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ST-58</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Home → challenge card → See challenges → Start Mindful moments.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Message "… started"; the card on Home shows it with its steps and 7 days left; other challenges can't be started meanwhile.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ST-59</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FR 3 (challenges, reward accuracy), FR 4, FR 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">With Mindful moments running: Support → box breathing 3 times (all four rounds), 5-4-3-2-1 grounding twice (reopen Support), read a mindfulness article.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Each step ticks off (tap a step to go to its place). After the last one: +40 XP, the Here and Now badge pop-up, Home says "Challenge complete!".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ST-60</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Start a challenge, then Leave challenge → Leave.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The challenge is gone from Home; XP and badges unchanged; another challenge can be started.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ST-61</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NFR 6, FR 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">With a challenge that has breathing: aeroplane mode on, do box breathing, then aeroplane mode off and Retry.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The breathing counts for the challenge once the phone is back online.</t>
+  </si>
+  <si>
     <t xml:space="preserve">System test summary</t>
   </si>
   <si>
@@ -874,6 +961,24 @@
     <t xml:space="preserve">Reminder is on in Profile.</t>
   </si>
   <si>
+    <t xml:space="preserve">T9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Start a 7-day challenge.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The challenge shows on Home.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Find what Chipu can wear and when new outfits unlock.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opens Rewards → Chipu's wardrobe.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Completion rate = done (easily or with difficulty) ÷ participants who tried. A common target is 78% or more per task.</t>
   </si>
   <si>
@@ -1123,7 +1228,7 @@
     <t xml:space="preserve">L5</t>
   </si>
   <si>
-    <t xml:space="preserve">The daily quests and streak encouraged me to check in.</t>
+    <t xml:space="preserve">The daily quests, challenges and streak encouraged me to check in.</t>
   </si>
   <si>
     <t xml:space="preserve">L6</t>
@@ -1154,6 +1259,18 @@
   </si>
   <si>
     <t xml:space="preserve">I would recommend MindQuest to a friend.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unlocking new outfits for Chipu made me want to level up.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rest days made missing a day feel less discouraging.</t>
   </si>
   <si>
     <t xml:space="preserve">"Not applicable" answers (e.g. L3 for people who only used English) are left out.</t>
@@ -1907,7 +2024,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I54"/>
+  <dimension ref="A1:I62"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -3169,9 +3286,193 @@
       <c r="H54" s="7"/>
       <c r="I54" s="7"/>
     </row>
+    <row r="55" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="B55" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="C55" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="D55" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="E55" s="6" t="s">
+        <v>241</v>
+      </c>
+      <c r="F55" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G55" s="7"/>
+      <c r="H55" s="7"/>
+      <c r="I55" s="7"/>
+    </row>
+    <row r="56" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="5" t="s">
+        <v>242</v>
+      </c>
+      <c r="B56" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="C56" s="6" t="s">
+        <v>243</v>
+      </c>
+      <c r="D56" s="6" t="s">
+        <v>244</v>
+      </c>
+      <c r="E56" s="6" t="s">
+        <v>245</v>
+      </c>
+      <c r="F56" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G56" s="7"/>
+      <c r="H56" s="7"/>
+      <c r="I56" s="7"/>
+    </row>
+    <row r="57" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="B57" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="C57" s="6" t="s">
+        <v>247</v>
+      </c>
+      <c r="D57" s="6" t="s">
+        <v>248</v>
+      </c>
+      <c r="E57" s="6" t="s">
+        <v>249</v>
+      </c>
+      <c r="F57" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G57" s="7"/>
+      <c r="H57" s="7"/>
+      <c r="I57" s="7"/>
+    </row>
+    <row r="58" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="B58" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="C58" s="6" t="s">
+        <v>247</v>
+      </c>
+      <c r="D58" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="E58" s="6" t="s">
+        <v>252</v>
+      </c>
+      <c r="F58" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G58" s="7"/>
+      <c r="H58" s="7"/>
+      <c r="I58" s="7"/>
+    </row>
+    <row r="59" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="5" t="s">
+        <v>253</v>
+      </c>
+      <c r="B59" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="C59" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="D59" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="E59" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="F59" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G59" s="7"/>
+      <c r="H59" s="7"/>
+      <c r="I59" s="7"/>
+    </row>
+    <row r="60" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="5" t="s">
+        <v>256</v>
+      </c>
+      <c r="B60" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="C60" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="D60" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="E60" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="F60" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G60" s="7"/>
+      <c r="H60" s="7"/>
+      <c r="I60" s="7"/>
+    </row>
+    <row r="61" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="5" t="s">
+        <v>260</v>
+      </c>
+      <c r="B61" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="C61" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="D61" s="6" t="s">
+        <v>261</v>
+      </c>
+      <c r="E61" s="6" t="s">
+        <v>262</v>
+      </c>
+      <c r="F61" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G61" s="7"/>
+      <c r="H61" s="7"/>
+      <c r="I61" s="7"/>
+    </row>
+    <row r="62" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="5" t="s">
+        <v>263</v>
+      </c>
+      <c r="B62" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="C62" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="D62" s="6" t="s">
+        <v>265</v>
+      </c>
+      <c r="E62" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="F62" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G62" s="7"/>
+      <c r="H62" s="7"/>
+      <c r="I62" s="7"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I54"/>
-  <conditionalFormatting sqref="F2:F54">
+  <autoFilter ref="A1:I62"/>
+  <conditionalFormatting sqref="F2:F62">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
       <formula>"Pass"</formula>
     </cfRule>
@@ -3183,7 +3484,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F2:F54" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F2:F62" type="list">
       <formula1>"Pass,Fail,Blocked,Not run"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -3214,7 +3515,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>238</v>
+        <v>267</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3222,33 +3523,33 @@
         <v>18</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>239</v>
+        <v>268</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>240</v>
+        <v>269</v>
       </c>
       <c r="B4" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$F$2:$F$54,A4)</f>
+        <f aca="false">COUNTIF('System tests'!$F$2:$F$62,A4)</f>
         <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>241</v>
+        <v>270</v>
       </c>
       <c r="B5" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$F$2:$F$54,A5)</f>
+        <f aca="false">COUNTIF('System tests'!$F$2:$F$62,A5)</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>242</v>
+        <v>271</v>
       </c>
       <c r="B6" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$F$2:$F$54,A6)</f>
+        <f aca="false">COUNTIF('System tests'!$F$2:$F$62,A6)</f>
         <v>0</v>
       </c>
     </row>
@@ -3257,22 +3558,22 @@
         <v>27</v>
       </c>
       <c r="B7" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$F$2:$F$54,A7)</f>
-        <v>53</v>
+        <f aca="false">COUNTIF('System tests'!$F$2:$F$62,A7)</f>
+        <v>61</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>243</v>
+        <v>272</v>
       </c>
       <c r="B8" s="5" t="n">
         <f aca="false">SUM(B4:B7)</f>
-        <v>53</v>
+        <v>61</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>244</v>
+        <v>273</v>
       </c>
       <c r="B9" s="9" t="str">
         <f aca="false">IF(B4+B5+B6=0,"-",B4/(B4+B5+B6))</f>
@@ -3284,22 +3585,22 @@
         <v>14</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>239</v>
+        <v>268</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>240</v>
+        <v>269</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>241</v>
+        <v>270</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>242</v>
+        <v>271</v>
       </c>
       <c r="F11" s="4" t="s">
         <v>27</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>245</v>
+        <v>274</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3307,23 +3608,23 @@
         <v>23</v>
       </c>
       <c r="B12" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$54,A12)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$62,A12)</f>
         <v>8</v>
       </c>
       <c r="C12" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A12,'System tests'!$F$2:$F$54,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A12,'System tests'!$F$2:$F$62,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D12" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A12,'System tests'!$F$2:$F$54,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A12,'System tests'!$F$2:$F$62,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E12" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A12,'System tests'!$F$2:$F$54,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A12,'System tests'!$F$2:$F$62,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F12" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A12,'System tests'!$F$2:$F$54,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A12,'System tests'!$F$2:$F$62,"Not run")</f>
         <v>8</v>
       </c>
       <c r="G12" s="10" t="str">
@@ -3336,23 +3637,23 @@
         <v>50</v>
       </c>
       <c r="B13" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$54,A13)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$62,A13)</f>
         <v>1</v>
       </c>
       <c r="C13" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A13,'System tests'!$F$2:$F$54,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A13,'System tests'!$F$2:$F$62,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D13" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A13,'System tests'!$F$2:$F$54,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A13,'System tests'!$F$2:$F$62,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E13" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A13,'System tests'!$F$2:$F$54,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A13,'System tests'!$F$2:$F$62,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F13" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A13,'System tests'!$F$2:$F$54,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A13,'System tests'!$F$2:$F$62,"Not run")</f>
         <v>1</v>
       </c>
       <c r="G13" s="10" t="str">
@@ -3365,23 +3666,23 @@
         <v>54</v>
       </c>
       <c r="B14" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$54,A14)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$62,A14)</f>
         <v>1</v>
       </c>
       <c r="C14" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A14,'System tests'!$F$2:$F$54,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A14,'System tests'!$F$2:$F$62,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D14" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A14,'System tests'!$F$2:$F$54,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A14,'System tests'!$F$2:$F$62,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E14" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A14,'System tests'!$F$2:$F$54,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A14,'System tests'!$F$2:$F$62,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F14" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A14,'System tests'!$F$2:$F$54,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A14,'System tests'!$F$2:$F$62,"Not run")</f>
         <v>1</v>
       </c>
       <c r="G14" s="10" t="str">
@@ -3394,23 +3695,23 @@
         <v>59</v>
       </c>
       <c r="B15" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$54,A15)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$62,A15)</f>
         <v>8</v>
       </c>
       <c r="C15" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A15,'System tests'!$F$2:$F$54,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A15,'System tests'!$F$2:$F$62,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D15" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A15,'System tests'!$F$2:$F$54,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A15,'System tests'!$F$2:$F$62,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E15" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A15,'System tests'!$F$2:$F$54,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A15,'System tests'!$F$2:$F$62,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F15" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A15,'System tests'!$F$2:$F$54,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A15,'System tests'!$F$2:$F$62,"Not run")</f>
         <v>8</v>
       </c>
       <c r="G15" s="10" t="str">
@@ -3423,23 +3724,23 @@
         <v>78</v>
       </c>
       <c r="B16" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$54,A16)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$62,A16)</f>
         <v>2</v>
       </c>
       <c r="C16" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A16,'System tests'!$F$2:$F$54,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A16,'System tests'!$F$2:$F$62,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D16" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A16,'System tests'!$F$2:$F$54,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A16,'System tests'!$F$2:$F$62,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E16" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A16,'System tests'!$F$2:$F$54,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A16,'System tests'!$F$2:$F$62,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F16" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A16,'System tests'!$F$2:$F$54,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A16,'System tests'!$F$2:$F$62,"Not run")</f>
         <v>2</v>
       </c>
       <c r="G16" s="10" t="str">
@@ -3452,23 +3753,23 @@
         <v>98</v>
       </c>
       <c r="B17" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$54,A17)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$62,A17)</f>
         <v>2</v>
       </c>
       <c r="C17" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A17,'System tests'!$F$2:$F$54,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A17,'System tests'!$F$2:$F$62,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D17" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A17,'System tests'!$F$2:$F$54,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A17,'System tests'!$F$2:$F$62,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E17" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A17,'System tests'!$F$2:$F$54,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A17,'System tests'!$F$2:$F$62,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F17" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A17,'System tests'!$F$2:$F$54,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A17,'System tests'!$F$2:$F$62,"Not run")</f>
         <v>2</v>
       </c>
       <c r="G17" s="10" t="str">
@@ -3481,23 +3782,23 @@
         <v>103</v>
       </c>
       <c r="B18" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$54,A18)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$62,A18)</f>
         <v>4</v>
       </c>
       <c r="C18" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A18,'System tests'!$F$2:$F$54,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A18,'System tests'!$F$2:$F$62,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D18" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A18,'System tests'!$F$2:$F$54,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A18,'System tests'!$F$2:$F$62,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E18" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A18,'System tests'!$F$2:$F$54,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A18,'System tests'!$F$2:$F$62,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F18" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A18,'System tests'!$F$2:$F$54,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A18,'System tests'!$F$2:$F$62,"Not run")</f>
         <v>4</v>
       </c>
       <c r="G18" s="10" t="str">
@@ -3510,24 +3811,24 @@
         <v>120</v>
       </c>
       <c r="B19" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$54,A19)</f>
-        <v>5</v>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$62,A19)</f>
+        <v>12</v>
       </c>
       <c r="C19" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A19,'System tests'!$F$2:$F$54,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A19,'System tests'!$F$2:$F$62,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D19" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A19,'System tests'!$F$2:$F$54,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A19,'System tests'!$F$2:$F$62,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E19" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A19,'System tests'!$F$2:$F$54,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A19,'System tests'!$F$2:$F$62,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F19" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A19,'System tests'!$F$2:$F$54,"Not run")</f>
-        <v>5</v>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A19,'System tests'!$F$2:$F$62,"Not run")</f>
+        <v>12</v>
       </c>
       <c r="G19" s="10" t="str">
         <f aca="false">IF(C19+D19+E19=0,"-",C19/(C19+D19+E19))</f>
@@ -3539,23 +3840,23 @@
         <v>136</v>
       </c>
       <c r="B20" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$54,A20)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$62,A20)</f>
         <v>1</v>
       </c>
       <c r="C20" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A20,'System tests'!$F$2:$F$54,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A20,'System tests'!$F$2:$F$62,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D20" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A20,'System tests'!$F$2:$F$54,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A20,'System tests'!$F$2:$F$62,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E20" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A20,'System tests'!$F$2:$F$54,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A20,'System tests'!$F$2:$F$62,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F20" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A20,'System tests'!$F$2:$F$54,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A20,'System tests'!$F$2:$F$62,"Not run")</f>
         <v>1</v>
       </c>
       <c r="G20" s="10" t="str">
@@ -3568,23 +3869,23 @@
         <v>141</v>
       </c>
       <c r="B21" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$54,A21)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$62,A21)</f>
         <v>2</v>
       </c>
       <c r="C21" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A21,'System tests'!$F$2:$F$54,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A21,'System tests'!$F$2:$F$62,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D21" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A21,'System tests'!$F$2:$F$54,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A21,'System tests'!$F$2:$F$62,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E21" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A21,'System tests'!$F$2:$F$54,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A21,'System tests'!$F$2:$F$62,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F21" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A21,'System tests'!$F$2:$F$54,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A21,'System tests'!$F$2:$F$62,"Not run")</f>
         <v>2</v>
       </c>
       <c r="G21" s="10" t="str">
@@ -3597,24 +3898,24 @@
         <v>150</v>
       </c>
       <c r="B22" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$54,A22)</f>
-        <v>5</v>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$62,A22)</f>
+        <v>6</v>
       </c>
       <c r="C22" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A22,'System tests'!$F$2:$F$54,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A22,'System tests'!$F$2:$F$62,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D22" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A22,'System tests'!$F$2:$F$54,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A22,'System tests'!$F$2:$F$62,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E22" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A22,'System tests'!$F$2:$F$54,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A22,'System tests'!$F$2:$F$62,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F22" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A22,'System tests'!$F$2:$F$54,"Not run")</f>
-        <v>5</v>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A22,'System tests'!$F$2:$F$62,"Not run")</f>
+        <v>6</v>
       </c>
       <c r="G22" s="10" t="str">
         <f aca="false">IF(C22+D22+E22=0,"-",C22/(C22+D22+E22))</f>
@@ -3626,23 +3927,23 @@
         <v>166</v>
       </c>
       <c r="B23" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$54,A23)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$62,A23)</f>
         <v>2</v>
       </c>
       <c r="C23" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A23,'System tests'!$F$2:$F$54,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A23,'System tests'!$F$2:$F$62,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D23" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A23,'System tests'!$F$2:$F$54,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A23,'System tests'!$F$2:$F$62,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E23" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A23,'System tests'!$F$2:$F$54,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A23,'System tests'!$F$2:$F$62,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F23" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A23,'System tests'!$F$2:$F$54,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A23,'System tests'!$F$2:$F$62,"Not run")</f>
         <v>2</v>
       </c>
       <c r="G23" s="10" t="str">
@@ -3655,23 +3956,23 @@
         <v>174</v>
       </c>
       <c r="B24" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$54,A24)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$62,A24)</f>
         <v>3</v>
       </c>
       <c r="C24" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A24,'System tests'!$F$2:$F$54,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A24,'System tests'!$F$2:$F$62,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D24" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A24,'System tests'!$F$2:$F$54,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A24,'System tests'!$F$2:$F$62,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E24" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A24,'System tests'!$F$2:$F$54,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A24,'System tests'!$F$2:$F$62,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F24" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A24,'System tests'!$F$2:$F$54,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A24,'System tests'!$F$2:$F$62,"Not run")</f>
         <v>3</v>
       </c>
       <c r="G24" s="10" t="str">
@@ -3684,23 +3985,23 @@
         <v>185</v>
       </c>
       <c r="B25" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$54,A25)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$62,A25)</f>
         <v>7</v>
       </c>
       <c r="C25" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A25,'System tests'!$F$2:$F$54,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A25,'System tests'!$F$2:$F$62,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D25" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A25,'System tests'!$F$2:$F$54,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A25,'System tests'!$F$2:$F$62,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E25" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A25,'System tests'!$F$2:$F$54,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A25,'System tests'!$F$2:$F$62,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F25" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A25,'System tests'!$F$2:$F$54,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A25,'System tests'!$F$2:$F$62,"Not run")</f>
         <v>7</v>
       </c>
       <c r="G25" s="10" t="str">
@@ -3713,23 +4014,23 @@
         <v>206</v>
       </c>
       <c r="B26" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$54,A26)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$62,A26)</f>
         <v>1</v>
       </c>
       <c r="C26" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A26,'System tests'!$F$2:$F$54,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A26,'System tests'!$F$2:$F$62,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D26" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A26,'System tests'!$F$2:$F$54,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A26,'System tests'!$F$2:$F$62,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E26" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A26,'System tests'!$F$2:$F$54,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A26,'System tests'!$F$2:$F$62,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F26" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A26,'System tests'!$F$2:$F$54,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A26,'System tests'!$F$2:$F$62,"Not run")</f>
         <v>1</v>
       </c>
       <c r="G26" s="10" t="str">
@@ -3742,23 +4043,23 @@
         <v>214</v>
       </c>
       <c r="B27" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$54,A27)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$62,A27)</f>
         <v>1</v>
       </c>
       <c r="C27" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A27,'System tests'!$F$2:$F$54,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A27,'System tests'!$F$2:$F$62,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D27" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A27,'System tests'!$F$2:$F$54,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A27,'System tests'!$F$2:$F$62,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E27" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A27,'System tests'!$F$2:$F$54,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A27,'System tests'!$F$2:$F$62,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F27" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$54,$A27,'System tests'!$F$2:$F$54,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A27,'System tests'!$F$2:$F$62,"Not run")</f>
         <v>1</v>
       </c>
       <c r="G27" s="10" t="str">
@@ -3782,7 +4083,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
@@ -3798,50 +4099,50 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>246</v>
+        <v>275</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>247</v>
+        <v>276</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>248</v>
+        <v>277</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>249</v>
+        <v>278</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>250</v>
+        <v>279</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>251</v>
+        <v>280</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>252</v>
+        <v>281</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>253</v>
+        <v>282</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>254</v>
+        <v>283</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>255</v>
+        <v>284</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>256</v>
+        <v>285</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>257</v>
+        <v>286</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>258</v>
+        <v>287</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>259</v>
+        <v>288</v>
       </c>
       <c r="D4" s="7"/>
       <c r="E4" s="7"/>
@@ -3862,13 +4163,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>260</v>
+        <v>289</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>261</v>
+        <v>290</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>262</v>
+        <v>291</v>
       </c>
       <c r="D5" s="7"/>
       <c r="E5" s="7"/>
@@ -3889,13 +4190,13 @@
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>263</v>
+        <v>292</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>264</v>
+        <v>293</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>265</v>
+        <v>294</v>
       </c>
       <c r="D6" s="7"/>
       <c r="E6" s="7"/>
@@ -3916,13 +4217,13 @@
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>266</v>
+        <v>295</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>267</v>
+        <v>296</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>268</v>
+        <v>297</v>
       </c>
       <c r="D7" s="7"/>
       <c r="E7" s="7"/>
@@ -3943,13 +4244,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>269</v>
+        <v>298</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>270</v>
+        <v>299</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>271</v>
+        <v>300</v>
       </c>
       <c r="D8" s="7"/>
       <c r="E8" s="7"/>
@@ -3970,13 +4271,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>272</v>
+        <v>301</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>273</v>
+        <v>302</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>274</v>
+        <v>303</v>
       </c>
       <c r="D9" s="7"/>
       <c r="E9" s="7"/>
@@ -3997,13 +4298,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>275</v>
+        <v>304</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>276</v>
+        <v>305</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>277</v>
+        <v>306</v>
       </c>
       <c r="D10" s="7"/>
       <c r="E10" s="7"/>
@@ -4024,13 +4325,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>278</v>
+        <v>307</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>279</v>
+        <v>308</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>280</v>
+        <v>309</v>
       </c>
       <c r="D11" s="7"/>
       <c r="E11" s="7"/>
@@ -4049,9 +4350,63 @@
         <v>-</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="12" t="s">
-        <v>281</v>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5" t="s">
+        <v>310</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>311</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>312</v>
+      </c>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="7"/>
+      <c r="H12" s="6" t="n">
+        <f aca="false">SUM(D12:G12)</f>
+        <v>0</v>
+      </c>
+      <c r="I12" s="10" t="str">
+        <f aca="false">IF(H12-G12&lt;=0,"-",(D12+E12)/(H12-G12))</f>
+        <v>-</v>
+      </c>
+      <c r="J12" s="10" t="str">
+        <f aca="false">IF(H12-G12&lt;=0,"-",D12/(H12-G12))</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="s">
+        <v>313</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>314</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>315</v>
+      </c>
+      <c r="D13" s="7"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="7"/>
+      <c r="H13" s="6" t="n">
+        <f aca="false">SUM(D13:G13)</f>
+        <v>0</v>
+      </c>
+      <c r="I13" s="10" t="str">
+        <f aca="false">IF(H13-G13&lt;=0,"-",(D13+E13)/(H13-G13))</f>
+        <v>-</v>
+      </c>
+      <c r="J13" s="10" t="str">
+        <f aca="false">IF(H13-G13&lt;=0,"-",D13/(H13-G13))</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="12" t="s">
+        <v>316</v>
       </c>
     </row>
   </sheetData>
@@ -4082,53 +4437,53 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>282</v>
+        <v>317</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>283</v>
+        <v>318</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>284</v>
+        <v>319</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>285</v>
+        <v>320</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>286</v>
+        <v>321</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>287</v>
+        <v>322</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>288</v>
+        <v>323</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>289</v>
+        <v>324</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>290</v>
+        <v>325</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>291</v>
+        <v>326</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>292</v>
+        <v>327</v>
       </c>
       <c r="K3" s="4" t="s">
-        <v>293</v>
+        <v>328</v>
       </c>
       <c r="L3" s="4" t="s">
-        <v>294</v>
+        <v>329</v>
       </c>
       <c r="N3" s="11" t="s">
-        <v>295</v>
+        <v>330</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>296</v>
+        <v>331</v>
       </c>
       <c r="B4" s="13" t="n">
         <v>4</v>
@@ -4165,7 +4520,7 @@
         <v>80</v>
       </c>
       <c r="N4" s="5" t="s">
-        <v>297</v>
+        <v>332</v>
       </c>
       <c r="O4" s="14" t="n">
         <f aca="false">COUNT(L5:L34)</f>
@@ -4174,7 +4529,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>298</v>
+        <v>333</v>
       </c>
       <c r="B5" s="7"/>
       <c r="C5" s="7"/>
@@ -4191,7 +4546,7 @@
         <v/>
       </c>
       <c r="N5" s="5" t="s">
-        <v>299</v>
+        <v>334</v>
       </c>
       <c r="O5" s="15" t="str">
         <f aca="false">IF(COUNT(L5:L34)=0,"-",AVERAGE(L5:L34))</f>
@@ -4200,7 +4555,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>300</v>
+        <v>335</v>
       </c>
       <c r="B6" s="7"/>
       <c r="C6" s="7"/>
@@ -4217,7 +4572,7 @@
         <v/>
       </c>
       <c r="N6" s="5" t="s">
-        <v>301</v>
+        <v>336</v>
       </c>
       <c r="O6" s="15" t="str">
         <f aca="false">IF(COUNT(L5:L34)=0,"-",MEDIAN(L5:L34))</f>
@@ -4226,7 +4581,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>302</v>
+        <v>337</v>
       </c>
       <c r="B7" s="7"/>
       <c r="C7" s="7"/>
@@ -4243,7 +4598,7 @@
         <v/>
       </c>
       <c r="N7" s="5" t="s">
-        <v>303</v>
+        <v>338</v>
       </c>
       <c r="O7" s="15" t="str">
         <f aca="false">IF(COUNT(L5:L34)&lt;2,"-",STDEV(L5:L34))</f>
@@ -4252,7 +4607,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>304</v>
+        <v>339</v>
       </c>
       <c r="B8" s="7"/>
       <c r="C8" s="7"/>
@@ -4269,7 +4624,7 @@
         <v/>
       </c>
       <c r="N8" s="5" t="s">
-        <v>305</v>
+        <v>340</v>
       </c>
       <c r="O8" s="15" t="str">
         <f aca="false">IF(COUNT(L5:L34)=0,"-",MIN(L5:L34))</f>
@@ -4278,7 +4633,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>306</v>
+        <v>341</v>
       </c>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
@@ -4295,7 +4650,7 @@
         <v/>
       </c>
       <c r="N9" s="5" t="s">
-        <v>307</v>
+        <v>342</v>
       </c>
       <c r="O9" s="15" t="str">
         <f aca="false">IF(COUNT(L5:L34)=0,"-",MAX(L5:L34))</f>
@@ -4304,7 +4659,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>308</v>
+        <v>343</v>
       </c>
       <c r="B10" s="7"/>
       <c r="C10" s="7"/>
@@ -4321,7 +4676,7 @@
         <v/>
       </c>
       <c r="N10" s="5" t="s">
-        <v>309</v>
+        <v>344</v>
       </c>
       <c r="O10" s="16" t="str">
         <f aca="false">IF(COUNT(L5:L34)=0,"-",IF(AVERAGE(L5:L34)&gt;68,"Yes","No"))</f>
@@ -4330,7 +4685,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>310</v>
+        <v>345</v>
       </c>
       <c r="B11" s="7"/>
       <c r="C11" s="7"/>
@@ -4349,7 +4704,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>311</v>
+        <v>346</v>
       </c>
       <c r="B12" s="7"/>
       <c r="C12" s="7"/>
@@ -4366,12 +4721,12 @@
         <v/>
       </c>
       <c r="N12" s="11" t="s">
-        <v>312</v>
+        <v>347</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>313</v>
+        <v>348</v>
       </c>
       <c r="B13" s="7"/>
       <c r="C13" s="7"/>
@@ -4388,12 +4743,12 @@
         <v/>
       </c>
       <c r="N13" s="17" t="s">
-        <v>314</v>
+        <v>349</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>315</v>
+        <v>350</v>
       </c>
       <c r="B14" s="7"/>
       <c r="C14" s="7"/>
@@ -4410,12 +4765,12 @@
         <v/>
       </c>
       <c r="N14" s="17" t="s">
-        <v>316</v>
+        <v>351</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>317</v>
+        <v>352</v>
       </c>
       <c r="B15" s="7"/>
       <c r="C15" s="7"/>
@@ -4432,12 +4787,12 @@
         <v/>
       </c>
       <c r="N15" s="17" t="s">
-        <v>318</v>
+        <v>353</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>319</v>
+        <v>354</v>
       </c>
       <c r="B16" s="7"/>
       <c r="C16" s="7"/>
@@ -4454,12 +4809,12 @@
         <v/>
       </c>
       <c r="N16" s="17" t="s">
-        <v>320</v>
+        <v>355</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>321</v>
+        <v>356</v>
       </c>
       <c r="B17" s="7"/>
       <c r="C17" s="7"/>
@@ -4476,12 +4831,12 @@
         <v/>
       </c>
       <c r="N17" s="17" t="s">
-        <v>322</v>
+        <v>357</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>323</v>
+        <v>358</v>
       </c>
       <c r="B18" s="7"/>
       <c r="C18" s="7"/>
@@ -4498,12 +4853,12 @@
         <v/>
       </c>
       <c r="N18" s="17" t="s">
-        <v>324</v>
+        <v>359</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>325</v>
+        <v>360</v>
       </c>
       <c r="B19" s="7"/>
       <c r="C19" s="7"/>
@@ -4520,12 +4875,12 @@
         <v/>
       </c>
       <c r="N19" s="17" t="s">
-        <v>326</v>
+        <v>361</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>327</v>
+        <v>362</v>
       </c>
       <c r="B20" s="7"/>
       <c r="C20" s="7"/>
@@ -4542,12 +4897,12 @@
         <v/>
       </c>
       <c r="N20" s="17" t="s">
-        <v>328</v>
+        <v>363</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>329</v>
+        <v>364</v>
       </c>
       <c r="B21" s="7"/>
       <c r="C21" s="7"/>
@@ -4564,12 +4919,12 @@
         <v/>
       </c>
       <c r="N21" s="17" t="s">
-        <v>330</v>
+        <v>365</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>331</v>
+        <v>366</v>
       </c>
       <c r="B22" s="7"/>
       <c r="C22" s="7"/>
@@ -4586,12 +4941,12 @@
         <v/>
       </c>
       <c r="N22" s="17" t="s">
-        <v>332</v>
+        <v>367</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>333</v>
+        <v>368</v>
       </c>
       <c r="B23" s="7"/>
       <c r="C23" s="7"/>
@@ -4610,7 +4965,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>334</v>
+        <v>369</v>
       </c>
       <c r="B24" s="7"/>
       <c r="C24" s="7"/>
@@ -4629,7 +4984,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>335</v>
+        <v>370</v>
       </c>
       <c r="B25" s="7"/>
       <c r="C25" s="7"/>
@@ -4648,7 +5003,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>336</v>
+        <v>371</v>
       </c>
       <c r="B26" s="7"/>
       <c r="C26" s="7"/>
@@ -4667,7 +5022,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
-        <v>337</v>
+        <v>372</v>
       </c>
       <c r="B27" s="7"/>
       <c r="C27" s="7"/>
@@ -4686,7 +5041,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
-        <v>338</v>
+        <v>373</v>
       </c>
       <c r="B28" s="7"/>
       <c r="C28" s="7"/>
@@ -4705,7 +5060,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
-        <v>339</v>
+        <v>374</v>
       </c>
       <c r="B29" s="7"/>
       <c r="C29" s="7"/>
@@ -4724,7 +5079,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
-        <v>340</v>
+        <v>375</v>
       </c>
       <c r="B30" s="7"/>
       <c r="C30" s="7"/>
@@ -4743,7 +5098,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
-        <v>341</v>
+        <v>376</v>
       </c>
       <c r="B31" s="7"/>
       <c r="C31" s="7"/>
@@ -4762,7 +5117,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
-        <v>342</v>
+        <v>377</v>
       </c>
       <c r="B32" s="7"/>
       <c r="C32" s="7"/>
@@ -4781,7 +5136,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
-        <v>343</v>
+        <v>378</v>
       </c>
       <c r="B33" s="7"/>
       <c r="C33" s="7"/>
@@ -4800,7 +5155,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
-        <v>344</v>
+        <v>379</v>
       </c>
       <c r="B34" s="7"/>
       <c r="C34" s="7"/>
@@ -4839,7 +5194,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -4852,47 +5207,47 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>345</v>
+        <v>380</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>346</v>
+        <v>381</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>347</v>
+        <v>382</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>348</v>
+        <v>383</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>349</v>
+        <v>384</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>350</v>
+        <v>385</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>351</v>
+        <v>386</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>352</v>
+        <v>387</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>254</v>
+        <v>283</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>353</v>
+        <v>388</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>354</v>
+        <v>389</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>355</v>
+        <v>390</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>356</v>
+        <v>391</v>
       </c>
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>
@@ -4914,10 +5269,10 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>357</v>
+        <v>392</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>358</v>
+        <v>393</v>
       </c>
       <c r="C5" s="7"/>
       <c r="D5" s="7"/>
@@ -4939,10 +5294,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>359</v>
+        <v>394</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>360</v>
+        <v>395</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="7"/>
@@ -4964,10 +5319,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>361</v>
+        <v>396</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>362</v>
+        <v>397</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
@@ -4987,12 +5342,12 @@
         <v>-</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>363</v>
+        <v>398</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>364</v>
+        <v>399</v>
       </c>
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
@@ -5014,10 +5369,10 @@
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>365</v>
+        <v>400</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>366</v>
+        <v>401</v>
       </c>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
@@ -5039,10 +5394,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>367</v>
+        <v>402</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>368</v>
+        <v>403</v>
       </c>
       <c r="C10" s="7"/>
       <c r="D10" s="7"/>
@@ -5064,10 +5419,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>369</v>
+        <v>404</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>370</v>
+        <v>405</v>
       </c>
       <c r="C11" s="7"/>
       <c r="D11" s="7"/>
@@ -5089,10 +5444,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>371</v>
+        <v>406</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>372</v>
+        <v>407</v>
       </c>
       <c r="C12" s="7"/>
       <c r="D12" s="7"/>
@@ -5114,10 +5469,10 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>373</v>
+        <v>408</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>374</v>
+        <v>409</v>
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="7"/>
@@ -5137,9 +5492,59 @@
         <v>-</v>
       </c>
     </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5" t="s">
+        <v>410</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>411</v>
+      </c>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="6" t="n">
+        <f aca="false">SUM(C14:G14)</f>
+        <v>0</v>
+      </c>
+      <c r="I14" s="10" t="str">
+        <f aca="false">IF(H14=0,"-",(F14+G14)/H14)</f>
+        <v>-</v>
+      </c>
+      <c r="J14" s="15" t="str">
+        <f aca="false">IF(H14=0,"-",(C14*1+D14*2+E14*3+F14*4+G14*5)/H14)</f>
+        <v>-</v>
+      </c>
+    </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="12" t="s">
-        <v>375</v>
+      <c r="A15" s="5" t="s">
+        <v>412</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>413</v>
+      </c>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="7"/>
+      <c r="H15" s="6" t="n">
+        <f aca="false">SUM(C15:G15)</f>
+        <v>0</v>
+      </c>
+      <c r="I15" s="10" t="str">
+        <f aca="false">IF(H15=0,"-",(F15+G15)/H15)</f>
+        <v>-</v>
+      </c>
+      <c r="J15" s="15" t="str">
+        <f aca="false">IF(H15=0,"-",(C15*1+D15*2+E15*3+F15*4+G15*5)/H15)</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="12" t="s">
+        <v>414</v>
       </c>
     </row>
   </sheetData>
@@ -5171,53 +5576,53 @@
   <sheetData>
     <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>376</v>
+        <v>415</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>377</v>
+        <v>416</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>378</v>
+        <v>417</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>379</v>
+        <v>418</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>380</v>
+        <v>419</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>381</v>
+        <v>420</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>382</v>
+        <v>421</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="13" t="s">
-        <v>296</v>
+        <v>331</v>
       </c>
       <c r="B2" s="13" t="s">
         <v>178</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>383</v>
+        <v>422</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>384</v>
+        <v>423</v>
       </c>
       <c r="E2" s="13" t="s">
-        <v>385</v>
+        <v>424</v>
       </c>
       <c r="F2" s="13" t="s">
-        <v>386</v>
+        <v>425</v>
       </c>
       <c r="G2" s="13" t="s">
-        <v>387</v>
+        <v>426</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>388</v>
+        <v>427</v>
       </c>
       <c r="B3" s="7"/>
       <c r="C3" s="7"/>
@@ -5228,7 +5633,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>389</v>
+        <v>428</v>
       </c>
       <c r="B4" s="7"/>
       <c r="C4" s="7"/>
@@ -5239,7 +5644,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>390</v>
+        <v>429</v>
       </c>
       <c r="B5" s="7"/>
       <c r="C5" s="7"/>
@@ -5250,7 +5655,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>391</v>
+        <v>430</v>
       </c>
       <c r="B6" s="7"/>
       <c r="C6" s="7"/>
@@ -5261,7 +5666,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>392</v>
+        <v>431</v>
       </c>
       <c r="B7" s="7"/>
       <c r="C7" s="7"/>
@@ -5272,7 +5677,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>393</v>
+        <v>432</v>
       </c>
       <c r="B8" s="7"/>
       <c r="C8" s="7"/>
@@ -5283,7 +5688,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>394</v>
+        <v>433</v>
       </c>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
@@ -5294,7 +5699,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>395</v>
+        <v>434</v>
       </c>
       <c r="B10" s="7"/>
       <c r="C10" s="7"/>
@@ -5305,7 +5710,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>396</v>
+        <v>435</v>
       </c>
       <c r="B11" s="7"/>
       <c r="C11" s="7"/>
@@ -5316,7 +5721,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>397</v>
+        <v>436</v>
       </c>
       <c r="B12" s="7"/>
       <c r="C12" s="7"/>
@@ -5327,7 +5732,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>398</v>
+        <v>437</v>
       </c>
       <c r="B13" s="7"/>
       <c r="C13" s="7"/>
@@ -5338,7 +5743,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>399</v>
+        <v>438</v>
       </c>
       <c r="B14" s="7"/>
       <c r="C14" s="7"/>
@@ -5349,7 +5754,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>400</v>
+        <v>439</v>
       </c>
       <c r="B15" s="7"/>
       <c r="C15" s="7"/>
@@ -5360,7 +5765,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>401</v>
+        <v>440</v>
       </c>
       <c r="B16" s="7"/>
       <c r="C16" s="7"/>
@@ -5371,7 +5776,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>402</v>
+        <v>441</v>
       </c>
       <c r="B17" s="7"/>
       <c r="C17" s="7"/>
@@ -5382,7 +5787,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>403</v>
+        <v>442</v>
       </c>
       <c r="B18" s="7"/>
       <c r="C18" s="7"/>
@@ -5393,7 +5798,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>404</v>
+        <v>443</v>
       </c>
       <c r="B19" s="7"/>
       <c r="C19" s="7"/>
@@ -5404,7 +5809,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>405</v>
+        <v>444</v>
       </c>
       <c r="B20" s="7"/>
       <c r="C20" s="7"/>
@@ -5415,7 +5820,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>406</v>
+        <v>445</v>
       </c>
       <c r="B21" s="7"/>
       <c r="C21" s="7"/>
@@ -5426,7 +5831,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>407</v>
+        <v>446</v>
       </c>
       <c r="B22" s="7"/>
       <c r="C22" s="7"/>
@@ -5437,7 +5842,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>408</v>
+        <v>447</v>
       </c>
       <c r="B23" s="7"/>
       <c r="C23" s="7"/>
@@ -5448,7 +5853,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>409</v>
+        <v>448</v>
       </c>
       <c r="B24" s="7"/>
       <c r="C24" s="7"/>
@@ -5459,7 +5864,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>410</v>
+        <v>449</v>
       </c>
       <c r="B25" s="7"/>
       <c r="C25" s="7"/>
@@ -5470,7 +5875,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>411</v>
+        <v>450</v>
       </c>
       <c r="B26" s="7"/>
       <c r="C26" s="7"/>
@@ -5481,7 +5886,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>412</v>
+        <v>451</v>
       </c>
       <c r="B27" s="7"/>
       <c r="C27" s="7"/>
@@ -5492,7 +5897,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
-        <v>413</v>
+        <v>452</v>
       </c>
       <c r="B28" s="7"/>
       <c r="C28" s="7"/>
@@ -5503,7 +5908,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>414</v>
+        <v>453</v>
       </c>
       <c r="B29" s="7"/>
       <c r="C29" s="7"/>
@@ -5514,7 +5919,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
-        <v>415</v>
+        <v>454</v>
       </c>
       <c r="B30" s="7"/>
       <c r="C30" s="7"/>
@@ -5525,7 +5930,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
-        <v>416</v>
+        <v>455</v>
       </c>
       <c r="B31" s="7"/>
       <c r="C31" s="7"/>
@@ -5536,7 +5941,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
-        <v>417</v>
+        <v>456</v>
       </c>
       <c r="B32" s="7"/>
       <c r="C32" s="7"/>

</xml_diff>

<commit_message>
Web version: big-screen layout, web sign-in, installable offline PWA, Netlify deploy
</commit_message>
<xml_diff>
--- a/docs/testing/MindQuest_testing.xlsx
+++ b/docs/testing/MindQuest_testing.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Bugs" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'System tests'!$A$1:$I$62</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'System tests'!$A$1:$I$67</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="605" uniqueCount="457">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="636" uniqueCount="476">
   <si>
     <t xml:space="preserve">MindQuest – testing workbook (step 12)</t>
   </si>
@@ -830,6 +830,63 @@
   </si>
   <si>
     <t xml:space="preserve">The breathing counts for the challenge once the phone is back online.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ST-62</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Web</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NFR 4, FR 6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open the website on a laptop in Chrome; sign in (Continue anonymously or Google). Visit every tab; switch the language.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loading screen, then the app; side menu on the left, pages in the middle at a readable width; Google sign-in comes back to the website; everything works as on the phone.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ST-63</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open the website on a phone browser; make the laptop browser window narrow.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bottom tabs as in the app; no text cut off.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ST-64</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NFR 6 (PWA caching)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">After one visit with internet, turn the internet off and reload the website (or open it again).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MindQuest still opens with the saved data and the offline banner; a check-in made now syncs when the internet is back.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ST-65</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NFR 4, NFR 6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chrome: Install app (address bar icon) or, on a phone, Add to Home screen. Open it from the icon.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Opens in its own window with the MindQuest name and icon.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ST-66</t>
+  </si>
+  <si>
+    <t xml:space="preserve">On the website, chat "I want to end it all"; tap Call on a helpline.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crisis sheet with helplines; on a phone the dialer opens; on a computer the number is shown and the browser offers a calling app.</t>
   </si>
   <si>
     <t xml:space="preserve">System test summary</t>
@@ -2024,7 +2081,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I62"/>
+  <dimension ref="A1:I67"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -3470,9 +3527,124 @@
       <c r="H62" s="7"/>
       <c r="I62" s="7"/>
     </row>
+    <row r="63" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="5" t="s">
+        <v>267</v>
+      </c>
+      <c r="B63" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="C63" s="6" t="s">
+        <v>269</v>
+      </c>
+      <c r="D63" s="6" t="s">
+        <v>270</v>
+      </c>
+      <c r="E63" s="6" t="s">
+        <v>271</v>
+      </c>
+      <c r="F63" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G63" s="7"/>
+      <c r="H63" s="7"/>
+      <c r="I63" s="7"/>
+    </row>
+    <row r="64" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="5" t="s">
+        <v>272</v>
+      </c>
+      <c r="B64" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="C64" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="D64" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="E64" s="6" t="s">
+        <v>274</v>
+      </c>
+      <c r="F64" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G64" s="7"/>
+      <c r="H64" s="7"/>
+      <c r="I64" s="7"/>
+    </row>
+    <row r="65" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="5" t="s">
+        <v>275</v>
+      </c>
+      <c r="B65" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="C65" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="D65" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="E65" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="F65" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G65" s="7"/>
+      <c r="H65" s="7"/>
+      <c r="I65" s="7"/>
+    </row>
+    <row r="66" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="B66" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="C66" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="D66" s="6" t="s">
+        <v>281</v>
+      </c>
+      <c r="E66" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="F66" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G66" s="7"/>
+      <c r="H66" s="7"/>
+      <c r="I66" s="7"/>
+    </row>
+    <row r="67" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="5" t="s">
+        <v>283</v>
+      </c>
+      <c r="B67" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="C67" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="D67" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="E67" s="6" t="s">
+        <v>285</v>
+      </c>
+      <c r="F67" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G67" s="7"/>
+      <c r="H67" s="7"/>
+      <c r="I67" s="7"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I62"/>
-  <conditionalFormatting sqref="F2:F62">
+  <autoFilter ref="A1:I67"/>
+  <conditionalFormatting sqref="F2:F67">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
       <formula>"Pass"</formula>
     </cfRule>
@@ -3484,7 +3656,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F2:F62" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F2:F67" type="list">
       <formula1>"Pass,Fail,Blocked,Not run"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -3505,7 +3677,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
@@ -3515,7 +3687,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>267</v>
+        <v>286</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3523,33 +3695,33 @@
         <v>18</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>268</v>
+        <v>287</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>269</v>
+        <v>288</v>
       </c>
       <c r="B4" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$F$2:$F$62,A4)</f>
+        <f aca="false">COUNTIF('System tests'!$F$2:$F$67,A4)</f>
         <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>270</v>
+        <v>289</v>
       </c>
       <c r="B5" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$F$2:$F$62,A5)</f>
+        <f aca="false">COUNTIF('System tests'!$F$2:$F$67,A5)</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>271</v>
+        <v>290</v>
       </c>
       <c r="B6" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$F$2:$F$62,A6)</f>
+        <f aca="false">COUNTIF('System tests'!$F$2:$F$67,A6)</f>
         <v>0</v>
       </c>
     </row>
@@ -3558,22 +3730,22 @@
         <v>27</v>
       </c>
       <c r="B7" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$F$2:$F$62,A7)</f>
-        <v>61</v>
+        <f aca="false">COUNTIF('System tests'!$F$2:$F$67,A7)</f>
+        <v>66</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>272</v>
+        <v>291</v>
       </c>
       <c r="B8" s="5" t="n">
         <f aca="false">SUM(B4:B7)</f>
-        <v>61</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>273</v>
+        <v>292</v>
       </c>
       <c r="B9" s="9" t="str">
         <f aca="false">IF(B4+B5+B6=0,"-",B4/(B4+B5+B6))</f>
@@ -3585,22 +3757,22 @@
         <v>14</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>268</v>
+        <v>287</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>269</v>
+        <v>288</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>270</v>
+        <v>289</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>271</v>
+        <v>290</v>
       </c>
       <c r="F11" s="4" t="s">
         <v>27</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>274</v>
+        <v>293</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3608,23 +3780,23 @@
         <v>23</v>
       </c>
       <c r="B12" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$62,A12)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$67,A12)</f>
         <v>8</v>
       </c>
       <c r="C12" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A12,'System tests'!$F$2:$F$62,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A12,'System tests'!$F$2:$F$67,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D12" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A12,'System tests'!$F$2:$F$62,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A12,'System tests'!$F$2:$F$67,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E12" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A12,'System tests'!$F$2:$F$62,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A12,'System tests'!$F$2:$F$67,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F12" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A12,'System tests'!$F$2:$F$62,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A12,'System tests'!$F$2:$F$67,"Not run")</f>
         <v>8</v>
       </c>
       <c r="G12" s="10" t="str">
@@ -3637,23 +3809,23 @@
         <v>50</v>
       </c>
       <c r="B13" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$62,A13)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$67,A13)</f>
         <v>1</v>
       </c>
       <c r="C13" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A13,'System tests'!$F$2:$F$62,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A13,'System tests'!$F$2:$F$67,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D13" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A13,'System tests'!$F$2:$F$62,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A13,'System tests'!$F$2:$F$67,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E13" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A13,'System tests'!$F$2:$F$62,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A13,'System tests'!$F$2:$F$67,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F13" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A13,'System tests'!$F$2:$F$62,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A13,'System tests'!$F$2:$F$67,"Not run")</f>
         <v>1</v>
       </c>
       <c r="G13" s="10" t="str">
@@ -3666,23 +3838,23 @@
         <v>54</v>
       </c>
       <c r="B14" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$62,A14)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$67,A14)</f>
         <v>1</v>
       </c>
       <c r="C14" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A14,'System tests'!$F$2:$F$62,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A14,'System tests'!$F$2:$F$67,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D14" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A14,'System tests'!$F$2:$F$62,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A14,'System tests'!$F$2:$F$67,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E14" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A14,'System tests'!$F$2:$F$62,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A14,'System tests'!$F$2:$F$67,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F14" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A14,'System tests'!$F$2:$F$62,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A14,'System tests'!$F$2:$F$67,"Not run")</f>
         <v>1</v>
       </c>
       <c r="G14" s="10" t="str">
@@ -3695,23 +3867,23 @@
         <v>59</v>
       </c>
       <c r="B15" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$62,A15)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$67,A15)</f>
         <v>8</v>
       </c>
       <c r="C15" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A15,'System tests'!$F$2:$F$62,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A15,'System tests'!$F$2:$F$67,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D15" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A15,'System tests'!$F$2:$F$62,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A15,'System tests'!$F$2:$F$67,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E15" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A15,'System tests'!$F$2:$F$62,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A15,'System tests'!$F$2:$F$67,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F15" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A15,'System tests'!$F$2:$F$62,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A15,'System tests'!$F$2:$F$67,"Not run")</f>
         <v>8</v>
       </c>
       <c r="G15" s="10" t="str">
@@ -3724,23 +3896,23 @@
         <v>78</v>
       </c>
       <c r="B16" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$62,A16)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$67,A16)</f>
         <v>2</v>
       </c>
       <c r="C16" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A16,'System tests'!$F$2:$F$62,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A16,'System tests'!$F$2:$F$67,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D16" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A16,'System tests'!$F$2:$F$62,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A16,'System tests'!$F$2:$F$67,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E16" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A16,'System tests'!$F$2:$F$62,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A16,'System tests'!$F$2:$F$67,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F16" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A16,'System tests'!$F$2:$F$62,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A16,'System tests'!$F$2:$F$67,"Not run")</f>
         <v>2</v>
       </c>
       <c r="G16" s="10" t="str">
@@ -3753,23 +3925,23 @@
         <v>98</v>
       </c>
       <c r="B17" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$62,A17)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$67,A17)</f>
         <v>2</v>
       </c>
       <c r="C17" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A17,'System tests'!$F$2:$F$62,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A17,'System tests'!$F$2:$F$67,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D17" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A17,'System tests'!$F$2:$F$62,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A17,'System tests'!$F$2:$F$67,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E17" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A17,'System tests'!$F$2:$F$62,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A17,'System tests'!$F$2:$F$67,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F17" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A17,'System tests'!$F$2:$F$62,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A17,'System tests'!$F$2:$F$67,"Not run")</f>
         <v>2</v>
       </c>
       <c r="G17" s="10" t="str">
@@ -3782,23 +3954,23 @@
         <v>103</v>
       </c>
       <c r="B18" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$62,A18)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$67,A18)</f>
         <v>4</v>
       </c>
       <c r="C18" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A18,'System tests'!$F$2:$F$62,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A18,'System tests'!$F$2:$F$67,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D18" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A18,'System tests'!$F$2:$F$62,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A18,'System tests'!$F$2:$F$67,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E18" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A18,'System tests'!$F$2:$F$62,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A18,'System tests'!$F$2:$F$67,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F18" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A18,'System tests'!$F$2:$F$62,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A18,'System tests'!$F$2:$F$67,"Not run")</f>
         <v>4</v>
       </c>
       <c r="G18" s="10" t="str">
@@ -3811,23 +3983,23 @@
         <v>120</v>
       </c>
       <c r="B19" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$62,A19)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$67,A19)</f>
         <v>12</v>
       </c>
       <c r="C19" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A19,'System tests'!$F$2:$F$62,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A19,'System tests'!$F$2:$F$67,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D19" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A19,'System tests'!$F$2:$F$62,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A19,'System tests'!$F$2:$F$67,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E19" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A19,'System tests'!$F$2:$F$62,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A19,'System tests'!$F$2:$F$67,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F19" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A19,'System tests'!$F$2:$F$62,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A19,'System tests'!$F$2:$F$67,"Not run")</f>
         <v>12</v>
       </c>
       <c r="G19" s="10" t="str">
@@ -3840,23 +4012,23 @@
         <v>136</v>
       </c>
       <c r="B20" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$62,A20)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$67,A20)</f>
         <v>1</v>
       </c>
       <c r="C20" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A20,'System tests'!$F$2:$F$62,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A20,'System tests'!$F$2:$F$67,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D20" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A20,'System tests'!$F$2:$F$62,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A20,'System tests'!$F$2:$F$67,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E20" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A20,'System tests'!$F$2:$F$62,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A20,'System tests'!$F$2:$F$67,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F20" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A20,'System tests'!$F$2:$F$62,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A20,'System tests'!$F$2:$F$67,"Not run")</f>
         <v>1</v>
       </c>
       <c r="G20" s="10" t="str">
@@ -3869,23 +4041,23 @@
         <v>141</v>
       </c>
       <c r="B21" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$62,A21)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$67,A21)</f>
         <v>2</v>
       </c>
       <c r="C21" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A21,'System tests'!$F$2:$F$62,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A21,'System tests'!$F$2:$F$67,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D21" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A21,'System tests'!$F$2:$F$62,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A21,'System tests'!$F$2:$F$67,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E21" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A21,'System tests'!$F$2:$F$62,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A21,'System tests'!$F$2:$F$67,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F21" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A21,'System tests'!$F$2:$F$62,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A21,'System tests'!$F$2:$F$67,"Not run")</f>
         <v>2</v>
       </c>
       <c r="G21" s="10" t="str">
@@ -3898,23 +4070,23 @@
         <v>150</v>
       </c>
       <c r="B22" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$62,A22)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$67,A22)</f>
         <v>6</v>
       </c>
       <c r="C22" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A22,'System tests'!$F$2:$F$62,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A22,'System tests'!$F$2:$F$67,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D22" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A22,'System tests'!$F$2:$F$62,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A22,'System tests'!$F$2:$F$67,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E22" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A22,'System tests'!$F$2:$F$62,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A22,'System tests'!$F$2:$F$67,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F22" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A22,'System tests'!$F$2:$F$62,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A22,'System tests'!$F$2:$F$67,"Not run")</f>
         <v>6</v>
       </c>
       <c r="G22" s="10" t="str">
@@ -3927,23 +4099,23 @@
         <v>166</v>
       </c>
       <c r="B23" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$62,A23)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$67,A23)</f>
         <v>2</v>
       </c>
       <c r="C23" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A23,'System tests'!$F$2:$F$62,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A23,'System tests'!$F$2:$F$67,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D23" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A23,'System tests'!$F$2:$F$62,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A23,'System tests'!$F$2:$F$67,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E23" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A23,'System tests'!$F$2:$F$62,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A23,'System tests'!$F$2:$F$67,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F23" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A23,'System tests'!$F$2:$F$62,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A23,'System tests'!$F$2:$F$67,"Not run")</f>
         <v>2</v>
       </c>
       <c r="G23" s="10" t="str">
@@ -3956,23 +4128,23 @@
         <v>174</v>
       </c>
       <c r="B24" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$62,A24)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$67,A24)</f>
         <v>3</v>
       </c>
       <c r="C24" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A24,'System tests'!$F$2:$F$62,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A24,'System tests'!$F$2:$F$67,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D24" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A24,'System tests'!$F$2:$F$62,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A24,'System tests'!$F$2:$F$67,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E24" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A24,'System tests'!$F$2:$F$62,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A24,'System tests'!$F$2:$F$67,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F24" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A24,'System tests'!$F$2:$F$62,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A24,'System tests'!$F$2:$F$67,"Not run")</f>
         <v>3</v>
       </c>
       <c r="G24" s="10" t="str">
@@ -3985,23 +4157,23 @@
         <v>185</v>
       </c>
       <c r="B25" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$62,A25)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$67,A25)</f>
         <v>7</v>
       </c>
       <c r="C25" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A25,'System tests'!$F$2:$F$62,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A25,'System tests'!$F$2:$F$67,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D25" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A25,'System tests'!$F$2:$F$62,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A25,'System tests'!$F$2:$F$67,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E25" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A25,'System tests'!$F$2:$F$62,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A25,'System tests'!$F$2:$F$67,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F25" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A25,'System tests'!$F$2:$F$62,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A25,'System tests'!$F$2:$F$67,"Not run")</f>
         <v>7</v>
       </c>
       <c r="G25" s="10" t="str">
@@ -4014,23 +4186,23 @@
         <v>206</v>
       </c>
       <c r="B26" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$62,A26)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$67,A26)</f>
         <v>1</v>
       </c>
       <c r="C26" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A26,'System tests'!$F$2:$F$62,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A26,'System tests'!$F$2:$F$67,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D26" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A26,'System tests'!$F$2:$F$62,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A26,'System tests'!$F$2:$F$67,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E26" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A26,'System tests'!$F$2:$F$62,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A26,'System tests'!$F$2:$F$67,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F26" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A26,'System tests'!$F$2:$F$62,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A26,'System tests'!$F$2:$F$67,"Not run")</f>
         <v>1</v>
       </c>
       <c r="G26" s="10" t="str">
@@ -4043,27 +4215,56 @@
         <v>214</v>
       </c>
       <c r="B27" s="6" t="n">
-        <f aca="false">COUNTIF('System tests'!$B$2:$B$62,A27)</f>
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$67,A27)</f>
         <v>1</v>
       </c>
       <c r="C27" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A27,'System tests'!$F$2:$F$62,"Pass")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A27,'System tests'!$F$2:$F$67,"Pass")</f>
         <v>0</v>
       </c>
       <c r="D27" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A27,'System tests'!$F$2:$F$62,"Fail")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A27,'System tests'!$F$2:$F$67,"Fail")</f>
         <v>0</v>
       </c>
       <c r="E27" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A27,'System tests'!$F$2:$F$62,"Blocked")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A27,'System tests'!$F$2:$F$67,"Blocked")</f>
         <v>0</v>
       </c>
       <c r="F27" s="6" t="n">
-        <f aca="false">COUNTIFS('System tests'!$B$2:$B$62,$A27,'System tests'!$F$2:$F$62,"Not run")</f>
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A27,'System tests'!$F$2:$F$67,"Not run")</f>
         <v>1</v>
       </c>
       <c r="G27" s="10" t="str">
         <f aca="false">IF(C27+D27+E27=0,"-",C27/(C27+D27+E27))</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="B28" s="6" t="n">
+        <f aca="false">COUNTIF('System tests'!$B$2:$B$67,A28)</f>
+        <v>5</v>
+      </c>
+      <c r="C28" s="6" t="n">
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A28,'System tests'!$F$2:$F$67,"Pass")</f>
+        <v>0</v>
+      </c>
+      <c r="D28" s="6" t="n">
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A28,'System tests'!$F$2:$F$67,"Fail")</f>
+        <v>0</v>
+      </c>
+      <c r="E28" s="6" t="n">
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A28,'System tests'!$F$2:$F$67,"Blocked")</f>
+        <v>0</v>
+      </c>
+      <c r="F28" s="6" t="n">
+        <f aca="false">COUNTIFS('System tests'!$B$2:$B$67,$A28,'System tests'!$F$2:$F$67,"Not run")</f>
+        <v>5</v>
+      </c>
+      <c r="G28" s="10" t="str">
+        <f aca="false">IF(C28+D28+E28=0,"-",C28/(C28+D28+E28))</f>
         <v>-</v>
       </c>
     </row>
@@ -4099,50 +4300,50 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>275</v>
+        <v>294</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>276</v>
+        <v>295</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>277</v>
+        <v>296</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>278</v>
+        <v>297</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>279</v>
+        <v>298</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>280</v>
+        <v>299</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>281</v>
+        <v>300</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>282</v>
+        <v>301</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>283</v>
+        <v>302</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>284</v>
+        <v>303</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>285</v>
+        <v>304</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>286</v>
+        <v>305</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>287</v>
+        <v>306</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>288</v>
+        <v>307</v>
       </c>
       <c r="D4" s="7"/>
       <c r="E4" s="7"/>
@@ -4163,13 +4364,13 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>289</v>
+        <v>308</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>290</v>
+        <v>309</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>291</v>
+        <v>310</v>
       </c>
       <c r="D5" s="7"/>
       <c r="E5" s="7"/>
@@ -4190,13 +4391,13 @@
     </row>
     <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>292</v>
+        <v>311</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>293</v>
+        <v>312</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>294</v>
+        <v>313</v>
       </c>
       <c r="D6" s="7"/>
       <c r="E6" s="7"/>
@@ -4217,13 +4418,13 @@
     </row>
     <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>295</v>
+        <v>314</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>296</v>
+        <v>315</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>297</v>
+        <v>316</v>
       </c>
       <c r="D7" s="7"/>
       <c r="E7" s="7"/>
@@ -4244,13 +4445,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>298</v>
+        <v>317</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>299</v>
+        <v>318</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>300</v>
+        <v>319</v>
       </c>
       <c r="D8" s="7"/>
       <c r="E8" s="7"/>
@@ -4271,13 +4472,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>301</v>
+        <v>320</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>302</v>
+        <v>321</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>303</v>
+        <v>322</v>
       </c>
       <c r="D9" s="7"/>
       <c r="E9" s="7"/>
@@ -4298,13 +4499,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>304</v>
+        <v>323</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>305</v>
+        <v>324</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>306</v>
+        <v>325</v>
       </c>
       <c r="D10" s="7"/>
       <c r="E10" s="7"/>
@@ -4325,13 +4526,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>307</v>
+        <v>326</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>308</v>
+        <v>327</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>309</v>
+        <v>328</v>
       </c>
       <c r="D11" s="7"/>
       <c r="E11" s="7"/>
@@ -4352,13 +4553,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>310</v>
+        <v>329</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>311</v>
+        <v>330</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>312</v>
+        <v>331</v>
       </c>
       <c r="D12" s="7"/>
       <c r="E12" s="7"/>
@@ -4379,13 +4580,13 @@
     </row>
     <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>313</v>
+        <v>332</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>314</v>
+        <v>333</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>315</v>
+        <v>334</v>
       </c>
       <c r="D13" s="7"/>
       <c r="E13" s="7"/>
@@ -4406,7 +4607,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="12" t="s">
-        <v>316</v>
+        <v>335</v>
       </c>
     </row>
   </sheetData>
@@ -4437,53 +4638,53 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>317</v>
+        <v>336</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>318</v>
+        <v>337</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>319</v>
+        <v>338</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>320</v>
+        <v>339</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>321</v>
+        <v>340</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>322</v>
+        <v>341</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>323</v>
+        <v>342</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>324</v>
+        <v>343</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>325</v>
+        <v>344</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>326</v>
+        <v>345</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>327</v>
+        <v>346</v>
       </c>
       <c r="K3" s="4" t="s">
-        <v>328</v>
+        <v>347</v>
       </c>
       <c r="L3" s="4" t="s">
-        <v>329</v>
+        <v>348</v>
       </c>
       <c r="N3" s="11" t="s">
-        <v>330</v>
+        <v>349</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>331</v>
+        <v>350</v>
       </c>
       <c r="B4" s="13" t="n">
         <v>4</v>
@@ -4520,7 +4721,7 @@
         <v>80</v>
       </c>
       <c r="N4" s="5" t="s">
-        <v>332</v>
+        <v>351</v>
       </c>
       <c r="O4" s="14" t="n">
         <f aca="false">COUNT(L5:L34)</f>
@@ -4529,7 +4730,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>333</v>
+        <v>352</v>
       </c>
       <c r="B5" s="7"/>
       <c r="C5" s="7"/>
@@ -4546,7 +4747,7 @@
         <v/>
       </c>
       <c r="N5" s="5" t="s">
-        <v>334</v>
+        <v>353</v>
       </c>
       <c r="O5" s="15" t="str">
         <f aca="false">IF(COUNT(L5:L34)=0,"-",AVERAGE(L5:L34))</f>
@@ -4555,7 +4756,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>335</v>
+        <v>354</v>
       </c>
       <c r="B6" s="7"/>
       <c r="C6" s="7"/>
@@ -4572,7 +4773,7 @@
         <v/>
       </c>
       <c r="N6" s="5" t="s">
-        <v>336</v>
+        <v>355</v>
       </c>
       <c r="O6" s="15" t="str">
         <f aca="false">IF(COUNT(L5:L34)=0,"-",MEDIAN(L5:L34))</f>
@@ -4581,7 +4782,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>337</v>
+        <v>356</v>
       </c>
       <c r="B7" s="7"/>
       <c r="C7" s="7"/>
@@ -4598,7 +4799,7 @@
         <v/>
       </c>
       <c r="N7" s="5" t="s">
-        <v>338</v>
+        <v>357</v>
       </c>
       <c r="O7" s="15" t="str">
         <f aca="false">IF(COUNT(L5:L34)&lt;2,"-",STDEV(L5:L34))</f>
@@ -4607,7 +4808,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>339</v>
+        <v>358</v>
       </c>
       <c r="B8" s="7"/>
       <c r="C8" s="7"/>
@@ -4624,7 +4825,7 @@
         <v/>
       </c>
       <c r="N8" s="5" t="s">
-        <v>340</v>
+        <v>359</v>
       </c>
       <c r="O8" s="15" t="str">
         <f aca="false">IF(COUNT(L5:L34)=0,"-",MIN(L5:L34))</f>
@@ -4633,7 +4834,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>341</v>
+        <v>360</v>
       </c>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
@@ -4650,7 +4851,7 @@
         <v/>
       </c>
       <c r="N9" s="5" t="s">
-        <v>342</v>
+        <v>361</v>
       </c>
       <c r="O9" s="15" t="str">
         <f aca="false">IF(COUNT(L5:L34)=0,"-",MAX(L5:L34))</f>
@@ -4659,7 +4860,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>343</v>
+        <v>362</v>
       </c>
       <c r="B10" s="7"/>
       <c r="C10" s="7"/>
@@ -4676,7 +4877,7 @@
         <v/>
       </c>
       <c r="N10" s="5" t="s">
-        <v>344</v>
+        <v>363</v>
       </c>
       <c r="O10" s="16" t="str">
         <f aca="false">IF(COUNT(L5:L34)=0,"-",IF(AVERAGE(L5:L34)&gt;68,"Yes","No"))</f>
@@ -4685,7 +4886,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>345</v>
+        <v>364</v>
       </c>
       <c r="B11" s="7"/>
       <c r="C11" s="7"/>
@@ -4704,7 +4905,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>346</v>
+        <v>365</v>
       </c>
       <c r="B12" s="7"/>
       <c r="C12" s="7"/>
@@ -4721,12 +4922,12 @@
         <v/>
       </c>
       <c r="N12" s="11" t="s">
-        <v>347</v>
+        <v>366</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>348</v>
+        <v>367</v>
       </c>
       <c r="B13" s="7"/>
       <c r="C13" s="7"/>
@@ -4743,12 +4944,12 @@
         <v/>
       </c>
       <c r="N13" s="17" t="s">
-        <v>349</v>
+        <v>368</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>350</v>
+        <v>369</v>
       </c>
       <c r="B14" s="7"/>
       <c r="C14" s="7"/>
@@ -4765,12 +4966,12 @@
         <v/>
       </c>
       <c r="N14" s="17" t="s">
-        <v>351</v>
+        <v>370</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>352</v>
+        <v>371</v>
       </c>
       <c r="B15" s="7"/>
       <c r="C15" s="7"/>
@@ -4787,12 +4988,12 @@
         <v/>
       </c>
       <c r="N15" s="17" t="s">
-        <v>353</v>
+        <v>372</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>354</v>
+        <v>373</v>
       </c>
       <c r="B16" s="7"/>
       <c r="C16" s="7"/>
@@ -4809,12 +5010,12 @@
         <v/>
       </c>
       <c r="N16" s="17" t="s">
-        <v>355</v>
+        <v>374</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>356</v>
+        <v>375</v>
       </c>
       <c r="B17" s="7"/>
       <c r="C17" s="7"/>
@@ -4831,12 +5032,12 @@
         <v/>
       </c>
       <c r="N17" s="17" t="s">
-        <v>357</v>
+        <v>376</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>358</v>
+        <v>377</v>
       </c>
       <c r="B18" s="7"/>
       <c r="C18" s="7"/>
@@ -4853,12 +5054,12 @@
         <v/>
       </c>
       <c r="N18" s="17" t="s">
-        <v>359</v>
+        <v>378</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>360</v>
+        <v>379</v>
       </c>
       <c r="B19" s="7"/>
       <c r="C19" s="7"/>
@@ -4875,12 +5076,12 @@
         <v/>
       </c>
       <c r="N19" s="17" t="s">
-        <v>361</v>
+        <v>380</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>362</v>
+        <v>381</v>
       </c>
       <c r="B20" s="7"/>
       <c r="C20" s="7"/>
@@ -4897,12 +5098,12 @@
         <v/>
       </c>
       <c r="N20" s="17" t="s">
-        <v>363</v>
+        <v>382</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>364</v>
+        <v>383</v>
       </c>
       <c r="B21" s="7"/>
       <c r="C21" s="7"/>
@@ -4919,12 +5120,12 @@
         <v/>
       </c>
       <c r="N21" s="17" t="s">
-        <v>365</v>
+        <v>384</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>366</v>
+        <v>385</v>
       </c>
       <c r="B22" s="7"/>
       <c r="C22" s="7"/>
@@ -4941,12 +5142,12 @@
         <v/>
       </c>
       <c r="N22" s="17" t="s">
-        <v>367</v>
+        <v>386</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>368</v>
+        <v>387</v>
       </c>
       <c r="B23" s="7"/>
       <c r="C23" s="7"/>
@@ -4965,7 +5166,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>369</v>
+        <v>388</v>
       </c>
       <c r="B24" s="7"/>
       <c r="C24" s="7"/>
@@ -4984,7 +5185,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>370</v>
+        <v>389</v>
       </c>
       <c r="B25" s="7"/>
       <c r="C25" s="7"/>
@@ -5003,7 +5204,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>371</v>
+        <v>390</v>
       </c>
       <c r="B26" s="7"/>
       <c r="C26" s="7"/>
@@ -5022,7 +5223,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
-        <v>372</v>
+        <v>391</v>
       </c>
       <c r="B27" s="7"/>
       <c r="C27" s="7"/>
@@ -5041,7 +5242,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
-        <v>373</v>
+        <v>392</v>
       </c>
       <c r="B28" s="7"/>
       <c r="C28" s="7"/>
@@ -5060,7 +5261,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
-        <v>374</v>
+        <v>393</v>
       </c>
       <c r="B29" s="7"/>
       <c r="C29" s="7"/>
@@ -5079,7 +5280,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
-        <v>375</v>
+        <v>394</v>
       </c>
       <c r="B30" s="7"/>
       <c r="C30" s="7"/>
@@ -5098,7 +5299,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
-        <v>376</v>
+        <v>395</v>
       </c>
       <c r="B31" s="7"/>
       <c r="C31" s="7"/>
@@ -5117,7 +5318,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
-        <v>377</v>
+        <v>396</v>
       </c>
       <c r="B32" s="7"/>
       <c r="C32" s="7"/>
@@ -5136,7 +5337,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
-        <v>378</v>
+        <v>397</v>
       </c>
       <c r="B33" s="7"/>
       <c r="C33" s="7"/>
@@ -5155,7 +5356,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
-        <v>379</v>
+        <v>398</v>
       </c>
       <c r="B34" s="7"/>
       <c r="C34" s="7"/>
@@ -5207,47 +5408,47 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="11" t="s">
-        <v>380</v>
+        <v>399</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>381</v>
+        <v>400</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>382</v>
+        <v>401</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>383</v>
+        <v>402</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>384</v>
+        <v>403</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>385</v>
+        <v>404</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>386</v>
+        <v>405</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>387</v>
+        <v>406</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>283</v>
+        <v>302</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>388</v>
+        <v>407</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>389</v>
+        <v>408</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>390</v>
+        <v>409</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>391</v>
+        <v>410</v>
       </c>
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>
@@ -5269,10 +5470,10 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>392</v>
+        <v>411</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>393</v>
+        <v>412</v>
       </c>
       <c r="C5" s="7"/>
       <c r="D5" s="7"/>
@@ -5294,10 +5495,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>394</v>
+        <v>413</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>395</v>
+        <v>414</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="7"/>
@@ -5319,10 +5520,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>396</v>
+        <v>415</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>397</v>
+        <v>416</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
@@ -5344,10 +5545,10 @@
     </row>
     <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>398</v>
+        <v>417</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>399</v>
+        <v>418</v>
       </c>
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
@@ -5369,10 +5570,10 @@
     </row>
     <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>400</v>
+        <v>419</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>401</v>
+        <v>420</v>
       </c>
       <c r="C9" s="7"/>
       <c r="D9" s="7"/>
@@ -5394,10 +5595,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>402</v>
+        <v>421</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>403</v>
+        <v>422</v>
       </c>
       <c r="C10" s="7"/>
       <c r="D10" s="7"/>
@@ -5419,10 +5620,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>404</v>
+        <v>423</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>405</v>
+        <v>424</v>
       </c>
       <c r="C11" s="7"/>
       <c r="D11" s="7"/>
@@ -5444,10 +5645,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>406</v>
+        <v>425</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>407</v>
+        <v>426</v>
       </c>
       <c r="C12" s="7"/>
       <c r="D12" s="7"/>
@@ -5469,10 +5670,10 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>408</v>
+        <v>427</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>409</v>
+        <v>428</v>
       </c>
       <c r="C13" s="7"/>
       <c r="D13" s="7"/>
@@ -5494,10 +5695,10 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>410</v>
+        <v>429</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>411</v>
+        <v>430</v>
       </c>
       <c r="C14" s="7"/>
       <c r="D14" s="7"/>
@@ -5519,10 +5720,10 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>412</v>
+        <v>431</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>413</v>
+        <v>432</v>
       </c>
       <c r="C15" s="7"/>
       <c r="D15" s="7"/>
@@ -5544,7 +5745,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="12" t="s">
-        <v>414</v>
+        <v>433</v>
       </c>
     </row>
   </sheetData>
@@ -5576,53 +5777,53 @@
   <sheetData>
     <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>415</v>
+        <v>434</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>416</v>
+        <v>435</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>417</v>
+        <v>436</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>418</v>
+        <v>437</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>419</v>
+        <v>438</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>420</v>
+        <v>439</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>421</v>
+        <v>440</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="13" t="s">
-        <v>331</v>
+        <v>350</v>
       </c>
       <c r="B2" s="13" t="s">
         <v>178</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>422</v>
+        <v>441</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>423</v>
+        <v>442</v>
       </c>
       <c r="E2" s="13" t="s">
-        <v>424</v>
+        <v>443</v>
       </c>
       <c r="F2" s="13" t="s">
-        <v>425</v>
+        <v>444</v>
       </c>
       <c r="G2" s="13" t="s">
-        <v>426</v>
+        <v>445</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>427</v>
+        <v>446</v>
       </c>
       <c r="B3" s="7"/>
       <c r="C3" s="7"/>
@@ -5633,7 +5834,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>428</v>
+        <v>447</v>
       </c>
       <c r="B4" s="7"/>
       <c r="C4" s="7"/>
@@ -5644,7 +5845,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>429</v>
+        <v>448</v>
       </c>
       <c r="B5" s="7"/>
       <c r="C5" s="7"/>
@@ -5655,7 +5856,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>430</v>
+        <v>449</v>
       </c>
       <c r="B6" s="7"/>
       <c r="C6" s="7"/>
@@ -5666,7 +5867,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>431</v>
+        <v>450</v>
       </c>
       <c r="B7" s="7"/>
       <c r="C7" s="7"/>
@@ -5677,7 +5878,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>432</v>
+        <v>451</v>
       </c>
       <c r="B8" s="7"/>
       <c r="C8" s="7"/>
@@ -5688,7 +5889,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>433</v>
+        <v>452</v>
       </c>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
@@ -5699,7 +5900,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>434</v>
+        <v>453</v>
       </c>
       <c r="B10" s="7"/>
       <c r="C10" s="7"/>
@@ -5710,7 +5911,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>435</v>
+        <v>454</v>
       </c>
       <c r="B11" s="7"/>
       <c r="C11" s="7"/>
@@ -5721,7 +5922,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>436</v>
+        <v>455</v>
       </c>
       <c r="B12" s="7"/>
       <c r="C12" s="7"/>
@@ -5732,7 +5933,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>437</v>
+        <v>456</v>
       </c>
       <c r="B13" s="7"/>
       <c r="C13" s="7"/>
@@ -5743,7 +5944,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>438</v>
+        <v>457</v>
       </c>
       <c r="B14" s="7"/>
       <c r="C14" s="7"/>
@@ -5754,7 +5955,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>439</v>
+        <v>458</v>
       </c>
       <c r="B15" s="7"/>
       <c r="C15" s="7"/>
@@ -5765,7 +5966,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>440</v>
+        <v>459</v>
       </c>
       <c r="B16" s="7"/>
       <c r="C16" s="7"/>
@@ -5776,7 +5977,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>441</v>
+        <v>460</v>
       </c>
       <c r="B17" s="7"/>
       <c r="C17" s="7"/>
@@ -5787,7 +5988,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>442</v>
+        <v>461</v>
       </c>
       <c r="B18" s="7"/>
       <c r="C18" s="7"/>
@@ -5798,7 +5999,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>443</v>
+        <v>462</v>
       </c>
       <c r="B19" s="7"/>
       <c r="C19" s="7"/>
@@ -5809,7 +6010,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>444</v>
+        <v>463</v>
       </c>
       <c r="B20" s="7"/>
       <c r="C20" s="7"/>
@@ -5820,7 +6021,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>445</v>
+        <v>464</v>
       </c>
       <c r="B21" s="7"/>
       <c r="C21" s="7"/>
@@ -5831,7 +6032,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>446</v>
+        <v>465</v>
       </c>
       <c r="B22" s="7"/>
       <c r="C22" s="7"/>
@@ -5842,7 +6043,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>447</v>
+        <v>466</v>
       </c>
       <c r="B23" s="7"/>
       <c r="C23" s="7"/>
@@ -5853,7 +6054,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>448</v>
+        <v>467</v>
       </c>
       <c r="B24" s="7"/>
       <c r="C24" s="7"/>
@@ -5864,7 +6065,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>449</v>
+        <v>468</v>
       </c>
       <c r="B25" s="7"/>
       <c r="C25" s="7"/>
@@ -5875,7 +6076,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>450</v>
+        <v>469</v>
       </c>
       <c r="B26" s="7"/>
       <c r="C26" s="7"/>
@@ -5886,7 +6087,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>451</v>
+        <v>470</v>
       </c>
       <c r="B27" s="7"/>
       <c r="C27" s="7"/>
@@ -5897,7 +6098,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
-        <v>452</v>
+        <v>471</v>
       </c>
       <c r="B28" s="7"/>
       <c r="C28" s="7"/>
@@ -5908,7 +6109,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>453</v>
+        <v>472</v>
       </c>
       <c r="B29" s="7"/>
       <c r="C29" s="7"/>
@@ -5919,7 +6120,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
-        <v>454</v>
+        <v>473</v>
       </c>
       <c r="B30" s="7"/>
       <c r="C30" s="7"/>
@@ -5930,7 +6131,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
-        <v>455</v>
+        <v>474</v>
       </c>
       <c r="B31" s="7"/>
       <c r="C31" s="7"/>
@@ -5941,7 +6142,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
-        <v>456</v>
+        <v>475</v>
       </c>
       <c r="B32" s="7"/>
       <c r="C32" s="7"/>

</xml_diff>